<commit_message>
Élasticité en régression 3 ans (SLOPE ln-ln) au lieu des 2 bouts 24→26
Réponse à « pourquoi seulement 2024 et 2026 » : le forward-elasticity utilise
désormais les 3 millésimes via une régression log-log =SLOPE(LN(leads);LN(budget))
sur 2024·2025·2026, avec les 3 années visibles dans les blocs ①, ③ et l'onglet
organique. Plus robuste au bruit. Sur ces données de démo (parfaitement
log-linéaires, 2025 pile sur la droite) le chiffre est identique aux 2 bouts —
la méthode devient défendable sur données réelles. Le back-test (bloc ②) reste
calibré 24→25 par construction (sa fenêtre exclut 2026).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
+++ b/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
@@ -865,7 +865,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Élasticité = LN(leads pay.26 ÷ leads pay.24) ÷ LN(budget26 ÷ budget24). Puis : leads gagnés → inscrits → CA, pour le Δ ci-dessus.</t>
+          <t>Élasticité = pente de régression de ln(leads payants) sur ln(budget acq), sur les 3 années 2024·2025·2026 (=SLOPE(LN;LN)) — pas seulement 2 bouts.</t>
         </is>
       </c>
     </row>
@@ -882,50 +882,60 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
+          <t>L.pay25</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
           <t>L.pay26</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Bud.24</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Bud.25</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>Bud.26</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>Élasticité</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Élasticité 3 ans</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>Leads 2026</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>Inscrits 2026</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="K13" s="12" t="inlineStr">
         <is>
           <t>Conv.</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="L13" s="12" t="inlineStr">
         <is>
           <t>Leads gagnés</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
+      <c r="M13" s="12" t="inlineStr">
         <is>
           <t>Inscrits gagnés</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
+      <c r="N13" s="12" t="inlineStr">
         <is>
           <t>CA gagné (+Δ)</t>
         </is>
@@ -941,38 +951,44 @@
         <v>377</v>
       </c>
       <c r="C14" s="14" t="n">
+        <v>399</v>
+      </c>
+      <c r="D14" s="14" t="n">
         <v>422</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="E14" s="15" t="n">
         <v>12543</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="F14" s="15" t="n">
+        <v>13798</v>
+      </c>
+      <c r="G14" s="15" t="n">
         <v>15178</v>
       </c>
-      <c r="F14" s="16">
-        <f>LN(C14/B14)/LN(E14/D14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="14" t="n">
+      <c r="H14" s="16">
+        <f>SLOPE(LN(B14:D14),LN(E14:G14))</f>
+        <v/>
+      </c>
+      <c r="I14" s="14" t="n">
         <v>680</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="J14" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="I14" s="17">
-        <f>H14/G14</f>
-        <v/>
-      </c>
-      <c r="J14" s="18">
-        <f>C14*((1+$B$6)^F14-1)</f>
-        <v/>
-      </c>
-      <c r="K14" s="18">
-        <f>J14*I14</f>
-        <v/>
-      </c>
-      <c r="L14" s="19">
-        <f>K14*$B$7</f>
+      <c r="K14" s="17">
+        <f>J14/I14</f>
+        <v/>
+      </c>
+      <c r="L14" s="18">
+        <f>D14*((1+$B$6)^H14-1)</f>
+        <v/>
+      </c>
+      <c r="M14" s="18">
+        <f>L14*K14</f>
+        <v/>
+      </c>
+      <c r="N14" s="19">
+        <f>M14*$B$7</f>
         <v/>
       </c>
     </row>
@@ -986,38 +1002,44 @@
         <v>489</v>
       </c>
       <c r="C15" s="14" t="n">
+        <v>516</v>
+      </c>
+      <c r="D15" s="14" t="n">
         <v>544</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="E15" s="15" t="n">
         <v>17983</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="F15" s="15" t="n">
+        <v>19782</v>
+      </c>
+      <c r="G15" s="15" t="n">
         <v>21760</v>
       </c>
-      <c r="F15" s="16">
-        <f>LN(C15/B15)/LN(E15/D15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="14" t="n">
+      <c r="H15" s="16">
+        <f>SLOPE(LN(B15:D15),LN(E15:G15))</f>
+        <v/>
+      </c>
+      <c r="I15" s="14" t="n">
         <v>850</v>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="J15" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="I15" s="17">
-        <f>H15/G15</f>
-        <v/>
-      </c>
-      <c r="J15" s="18">
-        <f>C15*((1+$B$6)^F15-1)</f>
-        <v/>
-      </c>
-      <c r="K15" s="18">
-        <f>J15*I15</f>
-        <v/>
-      </c>
-      <c r="L15" s="19">
-        <f>K15*$B$7</f>
+      <c r="K15" s="17">
+        <f>J15/I15</f>
+        <v/>
+      </c>
+      <c r="L15" s="18">
+        <f>D15*((1+$B$6)^H15-1)</f>
+        <v/>
+      </c>
+      <c r="M15" s="18">
+        <f>L15*K15</f>
+        <v/>
+      </c>
+      <c r="N15" s="19">
+        <f>M15*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1031,38 +1053,44 @@
         <v>371</v>
       </c>
       <c r="C16" s="14" t="n">
+        <v>392</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <v>415</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="E16" s="15" t="n">
         <v>12341</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="F16" s="15" t="n">
+        <v>13575</v>
+      </c>
+      <c r="G16" s="15" t="n">
         <v>14933</v>
       </c>
-      <c r="F16" s="16">
-        <f>LN(C16/B16)/LN(E16/D16)</f>
-        <v/>
-      </c>
-      <c r="G16" s="14" t="n">
+      <c r="H16" s="16">
+        <f>SLOPE(LN(B16:D16),LN(E16:G16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="14" t="n">
         <v>680</v>
       </c>
-      <c r="H16" s="14" t="n">
+      <c r="J16" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="I16" s="17">
-        <f>H16/G16</f>
-        <v/>
-      </c>
-      <c r="J16" s="18">
-        <f>C16*((1+$B$6)^F16-1)</f>
-        <v/>
-      </c>
-      <c r="K16" s="18">
-        <f>J16*I16</f>
-        <v/>
-      </c>
-      <c r="L16" s="19">
-        <f>K16*$B$7</f>
+      <c r="K16" s="17">
+        <f>J16/I16</f>
+        <v/>
+      </c>
+      <c r="L16" s="18">
+        <f>D16*((1+$B$6)^H16-1)</f>
+        <v/>
+      </c>
+      <c r="M16" s="18">
+        <f>L16*K16</f>
+        <v/>
+      </c>
+      <c r="N16" s="19">
+        <f>M16*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1076,38 +1104,44 @@
         <v>571</v>
       </c>
       <c r="C17" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <v>630</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="E17" s="15" t="n">
         <v>20843</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="F17" s="15" t="n">
+        <v>22927</v>
+      </c>
+      <c r="G17" s="15" t="n">
         <v>25220</v>
       </c>
-      <c r="F17" s="16">
-        <f>LN(C17/B17)/LN(E17/D17)</f>
-        <v/>
-      </c>
-      <c r="G17" s="14" t="n">
+      <c r="H17" s="16">
+        <f>SLOPE(LN(B17:D17),LN(E17:G17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="14" t="n">
         <v>1260</v>
       </c>
-      <c r="H17" s="14" t="n">
+      <c r="J17" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="I17" s="17">
-        <f>H17/G17</f>
-        <v/>
-      </c>
-      <c r="J17" s="18">
-        <f>C17*((1+$B$6)^F17-1)</f>
-        <v/>
-      </c>
-      <c r="K17" s="18">
-        <f>J17*I17</f>
-        <v/>
-      </c>
-      <c r="L17" s="19">
-        <f>K17*$B$7</f>
+      <c r="K17" s="17">
+        <f>J17/I17</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>D17*((1+$B$6)^H17-1)</f>
+        <v/>
+      </c>
+      <c r="M17" s="18">
+        <f>L17*K17</f>
+        <v/>
+      </c>
+      <c r="N17" s="19">
+        <f>M17*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1121,38 +1155,44 @@
         <v>1035</v>
       </c>
       <c r="C18" s="14" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <v>1126</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="E18" s="15" t="n">
         <v>50248</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="F18" s="15" t="n">
+        <v>55272</v>
+      </c>
+      <c r="G18" s="15" t="n">
         <v>60800</v>
       </c>
-      <c r="F18" s="16">
-        <f>LN(C18/B18)/LN(E18/D18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="14" t="n">
+      <c r="H18" s="16">
+        <f>SLOPE(LN(B18:D18),LN(E18:G18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="14" t="n">
         <v>1816</v>
       </c>
-      <c r="H18" s="14" t="n">
+      <c r="J18" s="14" t="n">
         <v>144</v>
       </c>
-      <c r="I18" s="17">
-        <f>H18/G18</f>
-        <v/>
-      </c>
-      <c r="J18" s="18">
-        <f>C18*((1+$B$6)^F18-1)</f>
-        <v/>
-      </c>
-      <c r="K18" s="18">
-        <f>J18*I18</f>
-        <v/>
-      </c>
-      <c r="L18" s="19">
-        <f>K18*$B$7</f>
+      <c r="K18" s="17">
+        <f>J18/I18</f>
+        <v/>
+      </c>
+      <c r="L18" s="18">
+        <f>D18*((1+$B$6)^H18-1)</f>
+        <v/>
+      </c>
+      <c r="M18" s="18">
+        <f>L18*K18</f>
+        <v/>
+      </c>
+      <c r="N18" s="19">
+        <f>M18*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1166,38 +1206,44 @@
         <v>526</v>
       </c>
       <c r="C19" s="14" t="n">
+        <v>553</v>
+      </c>
+      <c r="D19" s="14" t="n">
         <v>581</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="E19" s="15" t="n">
         <v>18251</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="F19" s="15" t="n">
+        <v>20076</v>
+      </c>
+      <c r="G19" s="15" t="n">
         <v>22083</v>
       </c>
-      <c r="F19" s="16">
-        <f>LN(C19/B19)/LN(E19/D19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="14" t="n">
+      <c r="H19" s="16">
+        <f>SLOPE(LN(B19:D19),LN(E19:G19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="14" t="n">
         <v>1186</v>
       </c>
-      <c r="H19" s="14" t="n">
+      <c r="J19" s="14" t="n">
         <v>94</v>
       </c>
-      <c r="I19" s="17">
-        <f>H19/G19</f>
-        <v/>
-      </c>
-      <c r="J19" s="18">
-        <f>C19*((1+$B$6)^F19-1)</f>
-        <v/>
-      </c>
-      <c r="K19" s="18">
-        <f>J19*I19</f>
-        <v/>
-      </c>
-      <c r="L19" s="19">
-        <f>K19*$B$7</f>
+      <c r="K19" s="17">
+        <f>J19/I19</f>
+        <v/>
+      </c>
+      <c r="L19" s="18">
+        <f>D19*((1+$B$6)^H19-1)</f>
+        <v/>
+      </c>
+      <c r="M19" s="18">
+        <f>L19*K19</f>
+        <v/>
+      </c>
+      <c r="N19" s="19">
+        <f>M19*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1211,38 +1257,44 @@
         <v>592</v>
       </c>
       <c r="C20" s="14" t="n">
+        <v>623</v>
+      </c>
+      <c r="D20" s="14" t="n">
         <v>656</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="E20" s="15" t="n">
         <v>20597</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="F20" s="15" t="n">
+        <v>22657</v>
+      </c>
+      <c r="G20" s="15" t="n">
         <v>24923</v>
       </c>
-      <c r="F20" s="16">
-        <f>LN(C20/B20)/LN(E20/D20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="14" t="n">
+      <c r="H20" s="16">
+        <f>SLOPE(LN(B20:D20),LN(E20:G20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="14" t="n">
         <v>1286</v>
       </c>
-      <c r="H20" s="14" t="n">
+      <c r="J20" s="14" t="n">
         <v>102</v>
       </c>
-      <c r="I20" s="17">
-        <f>H20/G20</f>
-        <v/>
-      </c>
-      <c r="J20" s="18">
-        <f>C20*((1+$B$6)^F20-1)</f>
-        <v/>
-      </c>
-      <c r="K20" s="18">
-        <f>J20*I20</f>
-        <v/>
-      </c>
-      <c r="L20" s="19">
-        <f>K20*$B$7</f>
+      <c r="K20" s="17">
+        <f>J20/I20</f>
+        <v/>
+      </c>
+      <c r="L20" s="18">
+        <f>D20*((1+$B$6)^H20-1)</f>
+        <v/>
+      </c>
+      <c r="M20" s="18">
+        <f>L20*K20</f>
+        <v/>
+      </c>
+      <c r="N20" s="19">
+        <f>M20*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1256,38 +1308,44 @@
         <v>863</v>
       </c>
       <c r="C21" s="14" t="n">
+        <v>905</v>
+      </c>
+      <c r="D21" s="14" t="n">
         <v>950</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="E21" s="15" t="n">
         <v>34532</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="F21" s="15" t="n">
+        <v>37985</v>
+      </c>
+      <c r="G21" s="15" t="n">
         <v>41783</v>
       </c>
-      <c r="F21" s="16">
-        <f>LN(C21/B21)/LN(E21/D21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="14" t="n">
+      <c r="H21" s="16">
+        <f>SLOPE(LN(B21:D21),LN(E21:G21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="14" t="n">
         <v>1666</v>
       </c>
-      <c r="H21" s="14" t="n">
+      <c r="J21" s="14" t="n">
         <v>132</v>
       </c>
-      <c r="I21" s="17">
-        <f>H21/G21</f>
-        <v/>
-      </c>
-      <c r="J21" s="18">
-        <f>C21*((1+$B$6)^F21-1)</f>
-        <v/>
-      </c>
-      <c r="K21" s="18">
-        <f>J21*I21</f>
-        <v/>
-      </c>
-      <c r="L21" s="19">
-        <f>K21*$B$7</f>
+      <c r="K21" s="17">
+        <f>J21/I21</f>
+        <v/>
+      </c>
+      <c r="L21" s="18">
+        <f>D21*((1+$B$6)^H21-1)</f>
+        <v/>
+      </c>
+      <c r="M21" s="18">
+        <f>L21*K21</f>
+        <v/>
+      </c>
+      <c r="N21" s="19">
+        <f>M21*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1301,38 +1359,44 @@
         <v>713</v>
       </c>
       <c r="C22" s="14" t="n">
+        <v>749</v>
+      </c>
+      <c r="D22" s="14" t="n">
         <v>788</v>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="E22" s="15" t="n">
         <v>26060</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="F22" s="15" t="n">
+        <v>28666</v>
+      </c>
+      <c r="G22" s="15" t="n">
         <v>31533</v>
       </c>
-      <c r="F22" s="16">
-        <f>LN(C22/B22)/LN(E22/D22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="14" t="n">
+      <c r="H22" s="16">
+        <f>SLOPE(LN(B22:D22),LN(E22:G22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="14" t="n">
         <v>1516</v>
       </c>
-      <c r="H22" s="14" t="n">
+      <c r="J22" s="14" t="n">
         <v>120</v>
       </c>
-      <c r="I22" s="17">
-        <f>H22/G22</f>
-        <v/>
-      </c>
-      <c r="J22" s="18">
-        <f>C22*((1+$B$6)^F22-1)</f>
-        <v/>
-      </c>
-      <c r="K22" s="18">
-        <f>J22*I22</f>
-        <v/>
-      </c>
-      <c r="L22" s="19">
-        <f>K22*$B$7</f>
+      <c r="K22" s="17">
+        <f>J22/I22</f>
+        <v/>
+      </c>
+      <c r="L22" s="18">
+        <f>D22*((1+$B$6)^H22-1)</f>
+        <v/>
+      </c>
+      <c r="M22" s="18">
+        <f>L22*K22</f>
+        <v/>
+      </c>
+      <c r="N22" s="19">
+        <f>M22*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1346,38 +1410,44 @@
         <v>1158</v>
       </c>
       <c r="C23" s="14" t="n">
+        <v>1210</v>
+      </c>
+      <c r="D23" s="14" t="n">
         <v>1265</v>
       </c>
-      <c r="D23" s="15" t="n">
+      <c r="E23" s="15" t="n">
         <v>56438</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="F23" s="15" t="n">
+        <v>62082</v>
+      </c>
+      <c r="G23" s="15" t="n">
         <v>68291</v>
       </c>
-      <c r="F23" s="16">
-        <f>LN(C23/B23)/LN(E23/D23)</f>
-        <v/>
-      </c>
-      <c r="G23" s="14" t="n">
+      <c r="H23" s="16">
+        <f>SLOPE(LN(B23:D23),LN(E23:G23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="14" t="n">
         <v>1976</v>
       </c>
-      <c r="H23" s="14" t="n">
+      <c r="J23" s="14" t="n">
         <v>156</v>
       </c>
-      <c r="I23" s="17">
-        <f>H23/G23</f>
-        <v/>
-      </c>
-      <c r="J23" s="18">
-        <f>C23*((1+$B$6)^F23-1)</f>
-        <v/>
-      </c>
-      <c r="K23" s="18">
-        <f>J23*I23</f>
-        <v/>
-      </c>
-      <c r="L23" s="19">
-        <f>K23*$B$7</f>
+      <c r="K23" s="17">
+        <f>J23/I23</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
+        <f>D23*((1+$B$6)^H23-1)</f>
+        <v/>
+      </c>
+      <c r="M23" s="18">
+        <f>L23*K23</f>
+        <v/>
+      </c>
+      <c r="N23" s="19">
+        <f>M23*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1391,38 +1461,44 @@
         <v>528</v>
       </c>
       <c r="C24" s="14" t="n">
+        <v>552</v>
+      </c>
+      <c r="D24" s="14" t="n">
         <v>578</v>
       </c>
-      <c r="D24" s="15" t="n">
+      <c r="E24" s="15" t="n">
         <v>18155</v>
       </c>
-      <c r="E24" s="15" t="n">
+      <c r="F24" s="15" t="n">
+        <v>19971</v>
+      </c>
+      <c r="G24" s="15" t="n">
         <v>21968</v>
       </c>
-      <c r="F24" s="16">
-        <f>LN(C24/B24)/LN(E24/D24)</f>
-        <v/>
-      </c>
-      <c r="G24" s="14" t="n">
+      <c r="H24" s="16">
+        <f>SLOPE(LN(B24:D24),LN(E24:G24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="14" t="n">
         <v>1230</v>
       </c>
-      <c r="H24" s="14" t="n">
+      <c r="J24" s="14" t="n">
         <v>72</v>
       </c>
-      <c r="I24" s="17">
-        <f>H24/G24</f>
-        <v/>
-      </c>
-      <c r="J24" s="18">
-        <f>C24*((1+$B$6)^F24-1)</f>
-        <v/>
-      </c>
-      <c r="K24" s="18">
-        <f>J24*I24</f>
-        <v/>
-      </c>
-      <c r="L24" s="19">
-        <f>K24*$B$7</f>
+      <c r="K24" s="17">
+        <f>J24/I24</f>
+        <v/>
+      </c>
+      <c r="L24" s="18">
+        <f>D24*((1+$B$6)^H24-1)</f>
+        <v/>
+      </c>
+      <c r="M24" s="18">
+        <f>L24*K24</f>
+        <v/>
+      </c>
+      <c r="N24" s="19">
+        <f>M24*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1436,38 +1512,44 @@
         <v>765</v>
       </c>
       <c r="C25" s="14" t="n">
+        <v>798</v>
+      </c>
+      <c r="D25" s="14" t="n">
         <v>832</v>
       </c>
-      <c r="D25" s="15" t="n">
+      <c r="E25" s="15" t="n">
         <v>30258</v>
       </c>
-      <c r="E25" s="15" t="n">
+      <c r="F25" s="15" t="n">
+        <v>33284</v>
+      </c>
+      <c r="G25" s="15" t="n">
         <v>36612</v>
       </c>
-      <c r="F25" s="16">
-        <f>LN(C25/B25)/LN(E25/D25)</f>
-        <v/>
-      </c>
-      <c r="G25" s="14" t="n">
+      <c r="H25" s="16">
+        <f>SLOPE(LN(B25:D25),LN(E25:G25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="14" t="n">
         <v>1570</v>
       </c>
-      <c r="H25" s="14" t="n">
+      <c r="J25" s="14" t="n">
         <v>92</v>
       </c>
-      <c r="I25" s="17">
-        <f>H25/G25</f>
-        <v/>
-      </c>
-      <c r="J25" s="18">
-        <f>C25*((1+$B$6)^F25-1)</f>
-        <v/>
-      </c>
-      <c r="K25" s="18">
-        <f>J25*I25</f>
-        <v/>
-      </c>
-      <c r="L25" s="19">
-        <f>K25*$B$7</f>
+      <c r="K25" s="17">
+        <f>J25/I25</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>D25*((1+$B$6)^H25-1)</f>
+        <v/>
+      </c>
+      <c r="M25" s="18">
+        <f>L25*K25</f>
+        <v/>
+      </c>
+      <c r="N25" s="19">
+        <f>M25*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1481,38 +1563,44 @@
         <v>392</v>
       </c>
       <c r="C26" s="14" t="n">
+        <v>410</v>
+      </c>
+      <c r="D26" s="14" t="n">
         <v>428</v>
       </c>
-      <c r="D26" s="15" t="n">
+      <c r="E26" s="15" t="n">
         <v>15578</v>
       </c>
-      <c r="E26" s="15" t="n">
+      <c r="F26" s="15" t="n">
+        <v>17136</v>
+      </c>
+      <c r="G26" s="15" t="n">
         <v>18850</v>
       </c>
-      <c r="F26" s="16">
-        <f>LN(C26/B26)/LN(E26/D26)</f>
-        <v/>
-      </c>
-      <c r="G26" s="14" t="n">
+      <c r="H26" s="16">
+        <f>SLOPE(LN(B26:D26),LN(E26:G26))</f>
+        <v/>
+      </c>
+      <c r="I26" s="14" t="n">
         <v>680</v>
       </c>
-      <c r="H26" s="14" t="n">
+      <c r="J26" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="I26" s="17">
-        <f>H26/G26</f>
-        <v/>
-      </c>
-      <c r="J26" s="18">
-        <f>C26*((1+$B$6)^F26-1)</f>
-        <v/>
-      </c>
-      <c r="K26" s="18">
-        <f>J26*I26</f>
-        <v/>
-      </c>
-      <c r="L26" s="19">
-        <f>K26*$B$7</f>
+      <c r="K26" s="17">
+        <f>J26/I26</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>D26*((1+$B$6)^H26-1)</f>
+        <v/>
+      </c>
+      <c r="M26" s="18">
+        <f>L26*K26</f>
+        <v/>
+      </c>
+      <c r="N26" s="19">
+        <f>M26*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1526,38 +1614,44 @@
         <v>517</v>
       </c>
       <c r="C27" s="14" t="n">
+        <v>538</v>
+      </c>
+      <c r="D27" s="14" t="n">
         <v>560</v>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="E27" s="15" t="n">
         <v>24992</v>
       </c>
-      <c r="E27" s="15" t="n">
+      <c r="F27" s="15" t="n">
+        <v>27491</v>
+      </c>
+      <c r="G27" s="15" t="n">
         <v>30240</v>
       </c>
-      <c r="F27" s="16">
-        <f>LN(C27/B27)/LN(E27/D27)</f>
-        <v/>
-      </c>
-      <c r="G27" s="14" t="n">
+      <c r="H27" s="16">
+        <f>SLOPE(LN(B27:D27),LN(E27:G27))</f>
+        <v/>
+      </c>
+      <c r="I27" s="14" t="n">
         <v>800</v>
       </c>
-      <c r="H27" s="14" t="n">
+      <c r="J27" s="14" t="n">
         <v>47</v>
       </c>
-      <c r="I27" s="17">
-        <f>H27/G27</f>
-        <v/>
-      </c>
-      <c r="J27" s="18">
-        <f>C27*((1+$B$6)^F27-1)</f>
-        <v/>
-      </c>
-      <c r="K27" s="18">
-        <f>J27*I27</f>
-        <v/>
-      </c>
-      <c r="L27" s="19">
-        <f>K27*$B$7</f>
+      <c r="K27" s="17">
+        <f>J27/I27</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>D27*((1+$B$6)^H27-1)</f>
+        <v/>
+      </c>
+      <c r="M27" s="18">
+        <f>L27*K27</f>
+        <v/>
+      </c>
+      <c r="N27" s="19">
+        <f>M27*$B$7</f>
         <v/>
       </c>
     </row>
@@ -1575,23 +1669,25 @@
       <c r="G28" s="21" t="n"/>
       <c r="H28" s="21" t="n"/>
       <c r="I28" s="21" t="n"/>
-      <c r="J28" s="22">
-        <f>SUM(J14:J27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="22">
-        <f>SUM(K14:K27)</f>
-        <v/>
-      </c>
-      <c r="L28" s="23">
+      <c r="J28" s="21" t="n"/>
+      <c r="K28" s="21" t="n"/>
+      <c r="L28" s="22">
         <f>SUM(L14:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="22">
+        <f>SUM(M14:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="23">
+        <f>SUM(N14:N27)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Cliquez « Élasticité » : =LN(…)/LN(…) sur les chiffres réels. Cliquez « CA gagné » : la chaîne complète jusqu'au CA.</t>
+          <t>Élasticité = régression sur 3 ans (robuste au bruit). Sur ces données 2025 est pile sur la droite → identique aux 2 bouts. Cliquez « CA gagné » : la chaîne jusqu'au CA.</t>
         </is>
       </c>
     </row>
@@ -2680,60 +2776,70 @@
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
+          <t>L.pay25</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
           <t>L.pay26</t>
         </is>
       </c>
-      <c r="D55" s="12" t="inlineStr">
+      <c r="E55" s="12" t="inlineStr">
         <is>
           <t>Bud.24</t>
         </is>
       </c>
-      <c r="E55" s="12" t="inlineStr">
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>Bud.25</t>
+        </is>
+      </c>
+      <c r="G55" s="12" t="inlineStr">
         <is>
           <t>Bud.26</t>
         </is>
       </c>
-      <c r="F55" s="12" t="inlineStr">
-        <is>
-          <t>Élasticité</t>
-        </is>
-      </c>
-      <c r="G55" s="12" t="inlineStr">
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>Élasticité 3 ans</t>
+        </is>
+      </c>
+      <c r="I55" s="12" t="inlineStr">
         <is>
           <t>Leads 2026</t>
         </is>
       </c>
-      <c r="H55" s="12" t="inlineStr">
+      <c r="J55" s="12" t="inlineStr">
         <is>
           <t>Inscrits 2026</t>
         </is>
       </c>
-      <c r="I55" s="12" t="inlineStr">
+      <c r="K55" s="12" t="inlineStr">
         <is>
           <t>Conv.</t>
         </is>
       </c>
-      <c r="J55" s="12" t="inlineStr">
+      <c r="L55" s="12" t="inlineStr">
         <is>
           <t>Δ budget</t>
         </is>
       </c>
-      <c r="K55" s="12" t="inlineStr">
+      <c r="M55" s="12" t="inlineStr">
         <is>
           <t>Inscrits gagnés</t>
         </is>
       </c>
-      <c r="L55" s="12" t="inlineStr">
+      <c r="N55" s="12" t="inlineStr">
         <is>
           <t>CA gagné</t>
         </is>
       </c>
-      <c r="M55" s="12" t="inlineStr">
+      <c r="O55" s="12" t="inlineStr">
         <is>
           <t>EBITDA gagné</t>
         </is>
       </c>
-      <c r="N55" s="12" t="inlineStr">
+      <c r="P55" s="12" t="inlineStr">
         <is>
           <t>CAC marg.</t>
         </is>
@@ -2749,46 +2855,52 @@
         <v>3326</v>
       </c>
       <c r="C56" s="14" t="n">
+        <v>3487</v>
+      </c>
+      <c r="D56" s="14" t="n">
         <v>3659</v>
       </c>
-      <c r="D56" s="14" t="n">
+      <c r="E56" s="14" t="n">
         <v>137627</v>
       </c>
-      <c r="E56" s="14" t="n">
+      <c r="F56" s="14" t="n">
+        <v>151390</v>
+      </c>
+      <c r="G56" s="14" t="n">
         <v>166530</v>
       </c>
-      <c r="F56" s="16">
-        <f>LN(C56/B56)/LN(E56/D56)</f>
-        <v/>
-      </c>
-      <c r="G56" s="14" t="n">
+      <c r="H56" s="16">
+        <f>SLOPE(LN(B56:D56),LN(E56:G56))</f>
+        <v/>
+      </c>
+      <c r="I56" s="14" t="n">
         <v>6444</v>
       </c>
-      <c r="H56" s="14" t="n">
+      <c r="J56" s="14" t="n">
         <v>510</v>
       </c>
-      <c r="I56" s="17">
-        <f>H56/G56</f>
-        <v/>
-      </c>
-      <c r="J56" s="36">
-        <f>E56*$B$6</f>
-        <v/>
-      </c>
-      <c r="K56" s="18">
-        <f>C56*((1+$B$6)^F56-1)*I56</f>
-        <v/>
-      </c>
-      <c r="L56" s="37">
-        <f>K56*$B$7</f>
-        <v/>
-      </c>
-      <c r="M56" s="38">
-        <f>L56-J56-K56*$B$8</f>
-        <v/>
-      </c>
-      <c r="N56" s="39">
-        <f>J56/K56</f>
+      <c r="K56" s="17">
+        <f>J56/I56</f>
+        <v/>
+      </c>
+      <c r="L56" s="36">
+        <f>G56*$B$6</f>
+        <v/>
+      </c>
+      <c r="M56" s="18">
+        <f>D56*((1+$B$6)^H56-1)*K56</f>
+        <v/>
+      </c>
+      <c r="N56" s="37">
+        <f>M56*$B$7</f>
+        <v/>
+      </c>
+      <c r="O56" s="38">
+        <f>N56-L56-M56*$B$8</f>
+        <v/>
+      </c>
+      <c r="P56" s="39">
+        <f>L56/M56</f>
         <v/>
       </c>
     </row>
@@ -2802,46 +2914,52 @@
         <v>2132</v>
       </c>
       <c r="C57" s="14" t="n">
+        <v>2233</v>
+      </c>
+      <c r="D57" s="14" t="n">
         <v>2337</v>
       </c>
-      <c r="D57" s="14" t="n">
+      <c r="E57" s="14" t="n">
         <v>89342</v>
       </c>
-      <c r="E57" s="14" t="n">
+      <c r="F57" s="14" t="n">
+        <v>98275</v>
+      </c>
+      <c r="G57" s="14" t="n">
         <v>108103</v>
       </c>
-      <c r="F57" s="16">
-        <f>LN(C57/B57)/LN(E57/D57)</f>
-        <v/>
-      </c>
-      <c r="G57" s="14" t="n">
+      <c r="H57" s="16">
+        <f>SLOPE(LN(B57:D57),LN(E57:G57))</f>
+        <v/>
+      </c>
+      <c r="I57" s="14" t="n">
         <v>4263</v>
       </c>
-      <c r="H57" s="14" t="n">
+      <c r="J57" s="14" t="n">
         <v>338</v>
       </c>
-      <c r="I57" s="17">
-        <f>H57/G57</f>
-        <v/>
-      </c>
-      <c r="J57" s="36">
-        <f>E57*$B$6</f>
-        <v/>
-      </c>
-      <c r="K57" s="18">
-        <f>C57*((1+$B$6)^F57-1)*I57</f>
-        <v/>
-      </c>
-      <c r="L57" s="37">
-        <f>K57*$B$7</f>
-        <v/>
-      </c>
-      <c r="M57" s="38">
-        <f>L57-J57-K57*$B$8</f>
-        <v/>
-      </c>
-      <c r="N57" s="39">
-        <f>J57/K57</f>
+      <c r="K57" s="17">
+        <f>J57/I57</f>
+        <v/>
+      </c>
+      <c r="L57" s="36">
+        <f>G57*$B$6</f>
+        <v/>
+      </c>
+      <c r="M57" s="18">
+        <f>D57*((1+$B$6)^H57-1)*K57</f>
+        <v/>
+      </c>
+      <c r="N57" s="37">
+        <f>M57*$B$7</f>
+        <v/>
+      </c>
+      <c r="O57" s="38">
+        <f>N57-L57-M57*$B$8</f>
+        <v/>
+      </c>
+      <c r="P57" s="39">
+        <f>L57/M57</f>
         <v/>
       </c>
     </row>
@@ -2855,46 +2973,52 @@
         <v>1237</v>
       </c>
       <c r="C58" s="14" t="n">
+        <v>1307</v>
+      </c>
+      <c r="D58" s="14" t="n">
         <v>1381</v>
       </c>
-      <c r="D58" s="14" t="n">
+      <c r="E58" s="14" t="n">
         <v>42867</v>
       </c>
-      <c r="E58" s="14" t="n">
+      <c r="F58" s="14" t="n">
+        <v>47155</v>
+      </c>
+      <c r="G58" s="14" t="n">
         <v>51871</v>
       </c>
-      <c r="F58" s="16">
-        <f>LN(C58/B58)/LN(E58/D58)</f>
-        <v/>
-      </c>
-      <c r="G58" s="14" t="n">
+      <c r="H58" s="16">
+        <f>SLOPE(LN(B58:D58),LN(E58:G58))</f>
+        <v/>
+      </c>
+      <c r="I58" s="14" t="n">
         <v>2210</v>
       </c>
-      <c r="H58" s="14" t="n">
+      <c r="J58" s="14" t="n">
         <v>130</v>
       </c>
-      <c r="I58" s="17">
-        <f>H58/G58</f>
-        <v/>
-      </c>
-      <c r="J58" s="36">
-        <f>E58*$B$6</f>
-        <v/>
-      </c>
-      <c r="K58" s="18">
-        <f>C58*((1+$B$6)^F58-1)*I58</f>
-        <v/>
-      </c>
-      <c r="L58" s="37">
-        <f>K58*$B$7</f>
-        <v/>
-      </c>
-      <c r="M58" s="38">
-        <f>L58-J58-K58*$B$8</f>
-        <v/>
-      </c>
-      <c r="N58" s="39">
-        <f>J58/K58</f>
+      <c r="K58" s="17">
+        <f>J58/I58</f>
+        <v/>
+      </c>
+      <c r="L58" s="36">
+        <f>G58*$B$6</f>
+        <v/>
+      </c>
+      <c r="M58" s="18">
+        <f>D58*((1+$B$6)^H58-1)*K58</f>
+        <v/>
+      </c>
+      <c r="N58" s="37">
+        <f>M58*$B$7</f>
+        <v/>
+      </c>
+      <c r="O58" s="38">
+        <f>N58-L58-M58*$B$8</f>
+        <v/>
+      </c>
+      <c r="P58" s="39">
+        <f>L58/M58</f>
         <v/>
       </c>
     </row>
@@ -2908,46 +3032,52 @@
         <v>1293</v>
       </c>
       <c r="C59" s="14" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D59" s="14" t="n">
         <v>1410</v>
       </c>
-      <c r="D59" s="14" t="n">
+      <c r="E59" s="14" t="n">
         <v>48413</v>
       </c>
-      <c r="E59" s="14" t="n">
+      <c r="F59" s="14" t="n">
+        <v>53255</v>
+      </c>
+      <c r="G59" s="14" t="n">
         <v>58580</v>
       </c>
-      <c r="F59" s="16">
-        <f>LN(C59/B59)/LN(E59/D59)</f>
-        <v/>
-      </c>
-      <c r="G59" s="14" t="n">
+      <c r="H59" s="16">
+        <f>SLOPE(LN(B59:D59),LN(E59:G59))</f>
+        <v/>
+      </c>
+      <c r="I59" s="14" t="n">
         <v>2800</v>
       </c>
-      <c r="H59" s="14" t="n">
+      <c r="J59" s="14" t="n">
         <v>164</v>
       </c>
-      <c r="I59" s="17">
-        <f>H59/G59</f>
-        <v/>
-      </c>
-      <c r="J59" s="36">
-        <f>E59*$B$6</f>
-        <v/>
-      </c>
-      <c r="K59" s="18">
-        <f>C59*((1+$B$6)^F59-1)*I59</f>
-        <v/>
-      </c>
-      <c r="L59" s="37">
-        <f>K59*$B$7</f>
-        <v/>
-      </c>
-      <c r="M59" s="38">
-        <f>L59-J59-K59*$B$8</f>
-        <v/>
-      </c>
-      <c r="N59" s="39">
-        <f>J59/K59</f>
+      <c r="K59" s="17">
+        <f>J59/I59</f>
+        <v/>
+      </c>
+      <c r="L59" s="36">
+        <f>G59*$B$6</f>
+        <v/>
+      </c>
+      <c r="M59" s="18">
+        <f>D59*((1+$B$6)^H59-1)*K59</f>
+        <v/>
+      </c>
+      <c r="N59" s="37">
+        <f>M59*$B$7</f>
+        <v/>
+      </c>
+      <c r="O59" s="38">
+        <f>N59-L59-M59*$B$8</f>
+        <v/>
+      </c>
+      <c r="P59" s="39">
+        <f>L59/M59</f>
         <v/>
       </c>
     </row>
@@ -2961,46 +3091,52 @@
         <v>909</v>
       </c>
       <c r="C60" s="14" t="n">
+        <v>948</v>
+      </c>
+      <c r="D60" s="14" t="n">
         <v>988</v>
       </c>
-      <c r="D60" s="14" t="n">
+      <c r="E60" s="14" t="n">
         <v>40570</v>
       </c>
-      <c r="E60" s="14" t="n">
+      <c r="F60" s="14" t="n">
+        <v>44627</v>
+      </c>
+      <c r="G60" s="14" t="n">
         <v>49090</v>
       </c>
-      <c r="F60" s="16">
-        <f>LN(C60/B60)/LN(E60/D60)</f>
-        <v/>
-      </c>
-      <c r="G60" s="14" t="n">
+      <c r="H60" s="16">
+        <f>SLOPE(LN(B60:D60),LN(E60:G60))</f>
+        <v/>
+      </c>
+      <c r="I60" s="14" t="n">
         <v>1480</v>
       </c>
-      <c r="H60" s="14" t="n">
+      <c r="J60" s="14" t="n">
         <v>87</v>
       </c>
-      <c r="I60" s="17">
-        <f>H60/G60</f>
-        <v/>
-      </c>
-      <c r="J60" s="36">
-        <f>E60*$B$6</f>
-        <v/>
-      </c>
-      <c r="K60" s="18">
-        <f>C60*((1+$B$6)^F60-1)*I60</f>
-        <v/>
-      </c>
-      <c r="L60" s="37">
-        <f>K60*$B$7</f>
-        <v/>
-      </c>
-      <c r="M60" s="38">
-        <f>L60-J60-K60*$B$8</f>
-        <v/>
-      </c>
-      <c r="N60" s="39">
-        <f>J60/K60</f>
+      <c r="K60" s="17">
+        <f>J60/I60</f>
+        <v/>
+      </c>
+      <c r="L60" s="36">
+        <f>G60*$B$6</f>
+        <v/>
+      </c>
+      <c r="M60" s="18">
+        <f>D60*((1+$B$6)^H60-1)*K60</f>
+        <v/>
+      </c>
+      <c r="N60" s="37">
+        <f>M60*$B$7</f>
+        <v/>
+      </c>
+      <c r="O60" s="38">
+        <f>N60-L60-M60*$B$8</f>
+        <v/>
+      </c>
+      <c r="P60" s="39">
+        <f>L60/M60</f>
         <v/>
       </c>
     </row>
@@ -3018,24 +3154,26 @@
       <c r="G61" s="21" t="n"/>
       <c r="H61" s="21" t="n"/>
       <c r="I61" s="21" t="n"/>
-      <c r="J61" s="41">
-        <f>SUM(J56:J60)</f>
-        <v/>
-      </c>
-      <c r="K61" s="42">
-        <f>SUM(K56:K60)</f>
-        <v/>
-      </c>
+      <c r="J61" s="21" t="n"/>
+      <c r="K61" s="21" t="n"/>
       <c r="L61" s="41">
         <f>SUM(L56:L60)</f>
         <v/>
       </c>
-      <c r="M61" s="41">
+      <c r="M61" s="42">
         <f>SUM(M56:M60)</f>
         <v/>
       </c>
-      <c r="N61" s="43">
-        <f>J61/K61</f>
+      <c r="N61" s="41">
+        <f>SUM(N56:N60)</f>
+        <v/>
+      </c>
+      <c r="O61" s="41">
+        <f>SUM(O56:O60)</f>
+        <v/>
+      </c>
+      <c r="P61" s="43">
+        <f>L61/M61</f>
         <v/>
       </c>
     </row>
@@ -3125,7 +3263,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Élasticité marque = LN(organiques 2026 ÷ organiques 2024) ÷ LN(budget marque 2026 ÷ budget marque 2024)</t>
+          <t>Élasticité marque = pente de régression de ln(organiques) sur ln(budget marque), sur 2024·2025·2026 (=SLOPE(LN;LN)).</t>
         </is>
       </c>
     </row>
@@ -3137,30 +3275,40 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Bud. marque 24</t>
+          <t>Bud.mq 24</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Bud. marque 26</t>
+          <t>Bud.mq 25</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
+          <t>Bud.mq 26</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
           <t>Organiques 24</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Organiques 25</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Organiques 26</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>Élasticité marque</t>
-        </is>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Élasticité marque 3 ans</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Org. gagnés (+Δ)</t>
         </is>
@@ -3176,20 +3324,26 @@
         <v>13581</v>
       </c>
       <c r="C12" s="15" t="n">
+        <v>17870</v>
+      </c>
+      <c r="D12" s="15" t="n">
         <v>23514</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="E12" s="14" t="n">
         <v>217</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="F12" s="14" t="n">
+        <v>237</v>
+      </c>
+      <c r="G12" s="14" t="n">
         <v>258</v>
       </c>
-      <c r="F12" s="16">
-        <f>LN(E12/D12)/LN(C12/B12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="18">
-        <f>E12*((1+$B$6)^F12-1)</f>
+      <c r="H12" s="16">
+        <f>SLOPE(LN(E12:G12),LN(B12:D12))</f>
+        <v/>
+      </c>
+      <c r="I12" s="18">
+        <f>G12*((1+$B$6)^H12-1)</f>
         <v/>
       </c>
     </row>
@@ -3203,20 +3357,26 @@
         <v>15937</v>
       </c>
       <c r="C13" s="15" t="n">
+        <v>21082</v>
+      </c>
+      <c r="D13" s="15" t="n">
         <v>27889</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="E13" s="14" t="n">
         <v>258</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="F13" s="14" t="n">
+        <v>281</v>
+      </c>
+      <c r="G13" s="14" t="n">
         <v>306</v>
       </c>
-      <c r="F13" s="16">
-        <f>LN(E13/D13)/LN(C13/B13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="18">
-        <f>E13*((1+$B$6)^F13-1)</f>
+      <c r="H13" s="16">
+        <f>SLOPE(LN(E13:G13),LN(B13:D13))</f>
+        <v/>
+      </c>
+      <c r="I13" s="18">
+        <f>G13*((1+$B$6)^H13-1)</f>
         <v/>
       </c>
     </row>
@@ -3230,20 +3390,26 @@
         <v>14022</v>
       </c>
       <c r="C14" s="15" t="n">
+        <v>18403</v>
+      </c>
+      <c r="D14" s="15" t="n">
         <v>24152</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="E14" s="14" t="n">
         <v>223</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="F14" s="14" t="n">
+        <v>243</v>
+      </c>
+      <c r="G14" s="14" t="n">
         <v>265</v>
       </c>
-      <c r="F14" s="16">
-        <f>LN(E14/D14)/LN(C14/B14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="18">
-        <f>E14*((1+$B$6)^F14-1)</f>
+      <c r="H14" s="16">
+        <f>SLOPE(LN(E14:G14),LN(B14:D14))</f>
+        <v/>
+      </c>
+      <c r="I14" s="18">
+        <f>G14*((1+$B$6)^H14-1)</f>
         <v/>
       </c>
     </row>
@@ -3257,20 +3423,26 @@
         <v>48495</v>
       </c>
       <c r="C15" s="15" t="n">
+        <v>52768</v>
+      </c>
+      <c r="D15" s="15" t="n">
         <v>57418</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="E15" s="14" t="n">
         <v>594</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="F15" s="14" t="n">
+        <v>612</v>
+      </c>
+      <c r="G15" s="14" t="n">
         <v>630</v>
       </c>
-      <c r="F15" s="16">
-        <f>LN(E15/D15)/LN(C15/B15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="18">
-        <f>E15*((1+$B$6)^F15-1)</f>
+      <c r="H15" s="16">
+        <f>SLOPE(LN(E15:G15),LN(B15:D15))</f>
+        <v/>
+      </c>
+      <c r="I15" s="18">
+        <f>G15*((1+$B$6)^H15-1)</f>
         <v/>
       </c>
     </row>
@@ -3284,20 +3456,26 @@
         <v>52094</v>
       </c>
       <c r="C16" s="15" t="n">
+        <v>57236</v>
+      </c>
+      <c r="D16" s="15" t="n">
         <v>62886</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="E16" s="14" t="n">
         <v>650</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="F16" s="14" t="n">
+        <v>670</v>
+      </c>
+      <c r="G16" s="14" t="n">
         <v>690</v>
       </c>
-      <c r="F16" s="16">
-        <f>LN(E16/D16)/LN(C16/B16)</f>
-        <v/>
-      </c>
-      <c r="G16" s="18">
-        <f>E16*((1+$B$6)^F16-1)</f>
+      <c r="H16" s="16">
+        <f>SLOPE(LN(E16:G16),LN(B16:D16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="18">
+        <f>G16*((1+$B$6)^H16-1)</f>
         <v/>
       </c>
     </row>
@@ -3311,20 +3489,26 @@
         <v>46637</v>
       </c>
       <c r="C17" s="15" t="n">
+        <v>50710</v>
+      </c>
+      <c r="D17" s="15" t="n">
         <v>55139</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="E17" s="14" t="n">
         <v>570</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="F17" s="14" t="n">
+        <v>587</v>
+      </c>
+      <c r="G17" s="14" t="n">
         <v>605</v>
       </c>
-      <c r="F17" s="16">
-        <f>LN(E17/D17)/LN(C17/B17)</f>
-        <v/>
-      </c>
-      <c r="G17" s="18">
-        <f>E17*((1+$B$6)^F17-1)</f>
+      <c r="H17" s="16">
+        <f>SLOPE(LN(E17:G17),LN(B17:D17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="18">
+        <f>G17*((1+$B$6)^H17-1)</f>
         <v/>
       </c>
     </row>
@@ -3338,20 +3522,26 @@
         <v>38877</v>
       </c>
       <c r="C18" s="15" t="n">
+        <v>47246</v>
+      </c>
+      <c r="D18" s="15" t="n">
         <v>57418</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="E18" s="14" t="n">
         <v>550</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="F18" s="14" t="n">
+        <v>589</v>
+      </c>
+      <c r="G18" s="14" t="n">
         <v>630</v>
       </c>
-      <c r="F18" s="16">
-        <f>LN(E18/D18)/LN(C18/B18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="18">
-        <f>E18*((1+$B$6)^F18-1)</f>
+      <c r="H18" s="16">
+        <f>SLOPE(LN(E18:G18),LN(B18:D18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="18">
+        <f>G18*((1+$B$6)^H18-1)</f>
         <v/>
       </c>
     </row>
@@ -3365,20 +3555,26 @@
         <v>43250</v>
       </c>
       <c r="C19" s="15" t="n">
+        <v>53125</v>
+      </c>
+      <c r="D19" s="15" t="n">
         <v>65255</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="E19" s="14" t="n">
         <v>626</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="F19" s="14" t="n">
+        <v>670</v>
+      </c>
+      <c r="G19" s="14" t="n">
         <v>716</v>
       </c>
-      <c r="F19" s="16">
-        <f>LN(E19/D19)/LN(C19/B19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="18">
-        <f>E19*((1+$B$6)^F19-1)</f>
+      <c r="H19" s="16">
+        <f>SLOPE(LN(E19:G19),LN(B19:D19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="18">
+        <f>G19*((1+$B$6)^H19-1)</f>
         <v/>
       </c>
     </row>
@@ -3392,20 +3588,26 @@
         <v>44771</v>
       </c>
       <c r="C20" s="15" t="n">
+        <v>54502</v>
+      </c>
+      <c r="D20" s="15" t="n">
         <v>66349</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="E20" s="14" t="n">
         <v>636</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="F20" s="14" t="n">
+        <v>680</v>
+      </c>
+      <c r="G20" s="14" t="n">
         <v>728</v>
       </c>
-      <c r="F20" s="16">
-        <f>LN(E20/D20)/LN(C20/B20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="18">
-        <f>E20*((1+$B$6)^F20-1)</f>
+      <c r="H20" s="16">
+        <f>SLOPE(LN(E20:G20),LN(B20:D20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="18">
+        <f>G20*((1+$B$6)^H20-1)</f>
         <v/>
       </c>
     </row>
@@ -3419,20 +3621,26 @@
         <v>41761</v>
       </c>
       <c r="C21" s="15" t="n">
+        <v>52020</v>
+      </c>
+      <c r="D21" s="15" t="n">
         <v>64800</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="E21" s="14" t="n">
         <v>621</v>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="F21" s="14" t="n">
+        <v>665</v>
+      </c>
+      <c r="G21" s="14" t="n">
         <v>711</v>
       </c>
-      <c r="F21" s="16">
-        <f>LN(E21/D21)/LN(C21/B21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="18">
-        <f>E21*((1+$B$6)^F21-1)</f>
+      <c r="H21" s="16">
+        <f>SLOPE(LN(E21:G21),LN(B21:D21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="18">
+        <f>G21*((1+$B$6)^H21-1)</f>
         <v/>
       </c>
     </row>
@@ -3446,20 +3654,26 @@
         <v>47760</v>
       </c>
       <c r="C22" s="15" t="n">
+        <v>53273</v>
+      </c>
+      <c r="D22" s="15" t="n">
         <v>59423</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="E22" s="14" t="n">
         <v>603</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="F22" s="14" t="n">
+        <v>627</v>
+      </c>
+      <c r="G22" s="14" t="n">
         <v>652</v>
       </c>
-      <c r="F22" s="16">
-        <f>LN(E22/D22)/LN(C22/B22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="18">
-        <f>E22*((1+$B$6)^F22-1)</f>
+      <c r="H22" s="16">
+        <f>SLOPE(LN(E22:G22),LN(B22:D22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="18">
+        <f>G22*((1+$B$6)^H22-1)</f>
         <v/>
       </c>
     </row>
@@ -3473,20 +3687,26 @@
         <v>53439</v>
       </c>
       <c r="C23" s="15" t="n">
+        <v>59953</v>
+      </c>
+      <c r="D23" s="15" t="n">
         <v>67261</v>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="E23" s="14" t="n">
         <v>682</v>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="F23" s="14" t="n">
+        <v>710</v>
+      </c>
+      <c r="G23" s="14" t="n">
         <v>738</v>
       </c>
-      <c r="F23" s="16">
-        <f>LN(E23/D23)/LN(C23/B23)</f>
-        <v/>
-      </c>
-      <c r="G23" s="18">
-        <f>E23*((1+$B$6)^F23-1)</f>
+      <c r="H23" s="16">
+        <f>SLOPE(LN(E23:G23),LN(B23:D23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="18">
+        <f>G23*((1+$B$6)^H23-1)</f>
         <v/>
       </c>
     </row>
@@ -3500,20 +3720,26 @@
         <v>20221</v>
       </c>
       <c r="C24" s="15" t="n">
+        <v>21550</v>
+      </c>
+      <c r="D24" s="15" t="n">
         <v>22967</v>
       </c>
-      <c r="D24" s="14" t="n">
+      <c r="E24" s="14" t="n">
         <v>242</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="F24" s="14" t="n">
+        <v>247</v>
+      </c>
+      <c r="G24" s="14" t="n">
         <v>252</v>
       </c>
-      <c r="F24" s="16">
-        <f>LN(E24/D24)/LN(C24/B24)</f>
-        <v/>
-      </c>
-      <c r="G24" s="18">
-        <f>E24*((1+$B$6)^F24-1)</f>
+      <c r="H24" s="16">
+        <f>SLOPE(LN(E24:G24),LN(B24:D24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="18">
+        <f>G24*((1+$B$6)^H24-1)</f>
         <v/>
       </c>
     </row>
@@ -3527,20 +3753,26 @@
         <v>19081</v>
       </c>
       <c r="C25" s="15" t="n">
+        <v>20429</v>
+      </c>
+      <c r="D25" s="15" t="n">
         <v>21873</v>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="E25" s="14" t="n">
         <v>231</v>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="F25" s="14" t="n">
+        <v>235</v>
+      </c>
+      <c r="G25" s="14" t="n">
         <v>240</v>
       </c>
-      <c r="F25" s="16">
-        <f>LN(E25/D25)/LN(C25/B25)</f>
-        <v/>
-      </c>
-      <c r="G25" s="18">
-        <f>E25*((1+$B$6)^F25-1)</f>
+      <c r="H25" s="16">
+        <f>SLOPE(LN(E25:G25),LN(B25:D25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="18">
+        <f>G25*((1+$B$6)^H25-1)</f>
         <v/>
       </c>
     </row>
@@ -3555,15 +3787,17 @@
       <c r="D26" s="21" t="n"/>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="21" t="n"/>
-      <c r="G26" s="22">
-        <f>SUM(G12:G25)</f>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="22">
+        <f>SUM(I12:I25)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Élasticité ~0,3 (vs ~0,5 pour l'acquisition) : le budget de marque agit, mais moins directement.</t>
+          <t>Élasticité ~0,3 (vs ~0,5 pour l'acquisition) : le budget de marque agit, mais moins directement. Régression sur 3 ans.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Back-test organique ajouté à l'onglet marque (symétrique de l'acquisition)
L'onglet « Budget de marque (organique) » a désormais son back-test : élasticité
marque calibrée 24→25, organiques 2026 prédits = org25 × (budmarque26/budmarque25)
^élast(24→25), comparés au réel. Prédit à +0,05 % au groupe (±0,4 % par campus).
Tout en formules cliquables.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
+++ b/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -180,6 +180,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="003D4F8F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00B3641C"/>
       <sz val="9"/>
     </font>
@@ -264,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -403,7 +409,16 @@
     <xf numFmtId="165" fontId="13" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="27" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2985,7 +3000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2997,6 +3012,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3557,10 +3573,619 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="48" t="inlineStr">
-        <is>
-          <t>Les deux leviers (acquisition + marque) alimentent le MÊME funnel → candidatures → inscrits → CA.</t>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>②  La preuve — back-test organique (calibré 24→25, prédit 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Élasticité marque calculée sur 2024→2025 seulement, puis : organiques 2026 prédits = org.25 × (budget marque 26 ÷ budget marque 25) ^ élasticité(24→25).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Campus</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Org.24</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Org.25</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Bud.mq24</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Bud.mq25</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Bud.mq26</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>Élast 24→25</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>Org.26 prédit</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Org.26 réel</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>Écart</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>Ipac Montpellier</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>217</v>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>237</v>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>13581</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>17870</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>23514</v>
+      </c>
+      <c r="G29" s="48">
+        <f>LN(C29/B29)/LN(E29/D29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="49">
+        <f>C29*(F29/E29)^G29</f>
+        <v/>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>258</v>
+      </c>
+      <c r="J29" s="50">
+        <f>H29/I29-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="46" t="inlineStr">
+        <is>
+          <t>Ipac Nantes</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>258</v>
+      </c>
+      <c r="C30" s="20" t="n">
+        <v>281</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>15937</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>21082</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>27889</v>
+      </c>
+      <c r="G30" s="48">
+        <f>LN(C30/B30)/LN(E30/D30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="49">
+        <f>C30*(F30/E30)^G30</f>
+        <v/>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>306</v>
+      </c>
+      <c r="J30" s="50">
+        <f>H30/I30-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="46" t="inlineStr">
+        <is>
+          <t>Ipac Rennes</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>223</v>
+      </c>
+      <c r="C31" s="20" t="n">
+        <v>243</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>14022</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>18403</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>24152</v>
+      </c>
+      <c r="G31" s="48">
+        <f>LN(C31/B31)/LN(E31/D31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="49">
+        <f>C31*(F31/E31)^G31</f>
+        <v/>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>265</v>
+      </c>
+      <c r="J31" s="50">
+        <f>H31/I31-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="46" t="inlineStr">
+        <is>
+          <t>Iscom Lille</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
+        <v>594</v>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>612</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>48495</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>52768</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <v>57418</v>
+      </c>
+      <c r="G32" s="48">
+        <f>LN(C32/B32)/LN(E32/D32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="49">
+        <f>C32*(F32/E32)^G32</f>
+        <v/>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>630</v>
+      </c>
+      <c r="J32" s="50">
+        <f>H32/I32-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="46" t="inlineStr">
+        <is>
+          <t>Iscom Paris</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
+        <v>650</v>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>670</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>52094</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>57236</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>62886</v>
+      </c>
+      <c r="G33" s="48">
+        <f>LN(C33/B33)/LN(E33/D33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="49">
+        <f>C33*(F33/E33)^G33</f>
+        <v/>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>690</v>
+      </c>
+      <c r="J33" s="50">
+        <f>H33/I33-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="46" t="inlineStr">
+        <is>
+          <t>Iscom Toulouse</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="n">
+        <v>570</v>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>587</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <v>46637</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>50710</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <v>55139</v>
+      </c>
+      <c r="G34" s="48">
+        <f>LN(C34/B34)/LN(E34/D34)</f>
+        <v/>
+      </c>
+      <c r="H34" s="49">
+        <f>C34*(F34/E34)^G34</f>
+        <v/>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>605</v>
+      </c>
+      <c r="J34" s="50">
+        <f>H34/I34-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>MBway Bordeaux</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
+        <v>550</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>589</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>38877</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>47246</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <v>57418</v>
+      </c>
+      <c r="G35" s="48">
+        <f>LN(C35/B35)/LN(E35/D35)</f>
+        <v/>
+      </c>
+      <c r="H35" s="49">
+        <f>C35*(F35/E35)^G35</f>
+        <v/>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>630</v>
+      </c>
+      <c r="J35" s="50">
+        <f>H35/I35-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>MBway Lyon</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
+        <v>626</v>
+      </c>
+      <c r="C36" s="20" t="n">
+        <v>670</v>
+      </c>
+      <c r="D36" s="20" t="n">
+        <v>43250</v>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>53125</v>
+      </c>
+      <c r="F36" s="20" t="n">
+        <v>65255</v>
+      </c>
+      <c r="G36" s="48">
+        <f>LN(C36/B36)/LN(E36/D36)</f>
+        <v/>
+      </c>
+      <c r="H36" s="49">
+        <f>C36*(F36/E36)^G36</f>
+        <v/>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>716</v>
+      </c>
+      <c r="J36" s="50">
+        <f>H36/I36-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>MBway Nantes</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
+        <v>636</v>
+      </c>
+      <c r="C37" s="20" t="n">
+        <v>680</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <v>44771</v>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>54502</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>66349</v>
+      </c>
+      <c r="G37" s="48">
+        <f>LN(C37/B37)/LN(E37/D37)</f>
+        <v/>
+      </c>
+      <c r="H37" s="49">
+        <f>C37*(F37/E37)^G37</f>
+        <v/>
+      </c>
+      <c r="I37" s="24" t="n">
+        <v>728</v>
+      </c>
+      <c r="J37" s="50">
+        <f>H37/I37-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="46" t="inlineStr">
+        <is>
+          <t>MBway Paris</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
+        <v>621</v>
+      </c>
+      <c r="C38" s="20" t="n">
+        <v>665</v>
+      </c>
+      <c r="D38" s="20" t="n">
+        <v>41761</v>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>52020</v>
+      </c>
+      <c r="F38" s="20" t="n">
+        <v>64800</v>
+      </c>
+      <c r="G38" s="48">
+        <f>LN(C38/B38)/LN(E38/D38)</f>
+        <v/>
+      </c>
+      <c r="H38" s="49">
+        <f>C38*(F38/E38)^G38</f>
+        <v/>
+      </c>
+      <c r="I38" s="24" t="n">
+        <v>711</v>
+      </c>
+      <c r="J38" s="50">
+        <f>H38/I38-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>Pigier Bordeaux</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>603</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <v>627</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>47760</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>53273</v>
+      </c>
+      <c r="F39" s="20" t="n">
+        <v>59423</v>
+      </c>
+      <c r="G39" s="48">
+        <f>LN(C39/B39)/LN(E39/D39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="49">
+        <f>C39*(F39/E39)^G39</f>
+        <v/>
+      </c>
+      <c r="I39" s="24" t="n">
+        <v>652</v>
+      </c>
+      <c r="J39" s="50">
+        <f>H39/I39-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="46" t="inlineStr">
+        <is>
+          <t>Pigier Lyon</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>682</v>
+      </c>
+      <c r="C40" s="20" t="n">
+        <v>710</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>53439</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>59953</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <v>67261</v>
+      </c>
+      <c r="G40" s="48">
+        <f>LN(C40/B40)/LN(E40/D40)</f>
+        <v/>
+      </c>
+      <c r="H40" s="49">
+        <f>C40*(F40/E40)^G40</f>
+        <v/>
+      </c>
+      <c r="I40" s="24" t="n">
+        <v>738</v>
+      </c>
+      <c r="J40" s="50">
+        <f>H40/I40-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="46" t="inlineStr">
+        <is>
+          <t>Tunon Lyon</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>242</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>247</v>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>20221</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <v>21550</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>22967</v>
+      </c>
+      <c r="G41" s="48">
+        <f>LN(C41/B41)/LN(E41/D41)</f>
+        <v/>
+      </c>
+      <c r="H41" s="49">
+        <f>C41*(F41/E41)^G41</f>
+        <v/>
+      </c>
+      <c r="I41" s="24" t="n">
+        <v>252</v>
+      </c>
+      <c r="J41" s="50">
+        <f>H41/I41-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>Tunon Paris</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>231</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>235</v>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>19081</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <v>20429</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>21873</v>
+      </c>
+      <c r="G42" s="48">
+        <f>LN(C42/B42)/LN(E42/D42)</f>
+        <v/>
+      </c>
+      <c r="H42" s="49">
+        <f>C42*(F42/E42)^G42</f>
+        <v/>
+      </c>
+      <c r="I42" s="24" t="n">
+        <v>240</v>
+      </c>
+      <c r="J42" s="50">
+        <f>H42/I42-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="43" t="inlineStr">
+        <is>
+          <t>GROUPE</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="29" t="n"/>
+      <c r="D43" s="29" t="n"/>
+      <c r="E43" s="29" t="n"/>
+      <c r="F43" s="29" t="n"/>
+      <c r="G43" s="29" t="n"/>
+      <c r="H43" s="44">
+        <f>SUM(H29:H42)</f>
+        <v/>
+      </c>
+      <c r="I43" s="44">
+        <f>SUM(I29:I42)</f>
+        <v/>
+      </c>
+      <c r="J43" s="45">
+        <f>H43/I43-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="51" t="inlineStr">
+        <is>
+          <t>Le moteur retrouve aussi les organiques 2026 sans les avoir vus. Les deux leviers (acquisition + marque) alimentent le MÊME funnel → inscrits → CA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Moteur : remplir les lignes agrégées (marque/groupe) du 1er tableau
Les sous-totaux marque et la ligne groupe n'affichaient que l'effet (additif) ;
les colonnes calibration restaient vides. On remplit désormais les volumes
(leads/budgets = somme) et la conversion (moyenne pondérée réelle Σinscrits÷Σleads).
Seule l'élasticité reste « — » : elle est propre à chaque campus et ne s'agrège
pas (on ne somme pas une élasticité). Régénère aussi le classeur final.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
+++ b/eduservices/tagetik/LE_MOTEUR_MODELE.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,6 +140,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="0051606D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007D8B98"/>
       <sz val="11"/>
     </font>
     <font>
@@ -280,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -318,10 +323,18 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -367,52 +380,61 @@
     <xf numFmtId="0" fontId="19" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="20" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="20" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="19" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="19" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="22" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="24" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="27" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="28" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="24" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="25" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="29" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -425,13 +447,13 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="29" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="30" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -977,263 +999,283 @@
           <t>MBway</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="B13" s="13">
+        <f>SUM(B14:B17)</f>
+        <v/>
+      </c>
+      <c r="C13" s="13">
+        <f>SUM(C14:C17)</f>
+        <v/>
+      </c>
+      <c r="D13" s="13">
+        <f>SUM(D14:D17)</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>SUM(E14:E17)</f>
+        <v/>
+      </c>
+      <c r="F13" s="14">
+        <f>SUM(F14:F17)</f>
+        <v/>
+      </c>
+      <c r="G13" s="14">
+        <f>SUM(G14:G17)</f>
+        <v/>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="15">
+      <c r="I13" s="16" t="n">
+        <v>0.07914338919925512</v>
+      </c>
+      <c r="J13" s="17">
         <f>M13/L13</f>
         <v/>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="18">
         <f>SUM(K14:K17)</f>
         <v/>
       </c>
-      <c r="L13" s="17">
+      <c r="L13" s="19">
         <f>SUM(L14:L17)</f>
         <v/>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="18">
         <f>SUM(M14:M17)</f>
         <v/>
       </c>
-      <c r="N13" s="16">
+      <c r="N13" s="18">
         <f>SUM(N14:N17)</f>
         <v/>
       </c>
-      <c r="O13" s="18">
+      <c r="O13" s="20">
         <f>K13/L13</f>
         <v/>
       </c>
     </row>
     <row r="14" hidden="1" outlineLevel="1">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n">
+      <c r="B14" s="22" t="n">
         <v>592</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <v>623</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="22" t="n">
         <v>656</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="22" t="n">
         <v>20597</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="22" t="n">
         <v>22657</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="22" t="n">
         <v>24923</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="23">
         <f>SLOPE(LN(B14:D14),LN(E14:G14))</f>
         <v/>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="24">
         <f>102/1286</f>
         <v/>
       </c>
-      <c r="J14" s="23" t="n">
+      <c r="J14" s="25" t="n">
         <v>7365</v>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="26">
         <f>G14*$B$6</f>
         <v/>
       </c>
-      <c r="L14" s="25">
+      <c r="L14" s="27">
         <f>D14*((1+$B$6)^H14-1)*I14</f>
         <v/>
       </c>
-      <c r="M14" s="26">
+      <c r="M14" s="28">
         <f>L14*J14</f>
         <v/>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="29">
         <f>M14-K14-L14*$B$7</f>
         <v/>
       </c>
-      <c r="O14" s="28">
+      <c r="O14" s="30">
         <f>K14/L14</f>
         <v/>
       </c>
     </row>
     <row r="15" hidden="1" outlineLevel="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n">
+      <c r="B15" s="22" t="n">
         <v>863</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <v>905</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="22" t="n">
         <v>950</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="22" t="n">
         <v>34532</v>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="22" t="n">
         <v>37985</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="G15" s="22" t="n">
         <v>41783</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="23">
         <f>SLOPE(LN(B15:D15),LN(E15:G15))</f>
         <v/>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="24">
         <f>132/1666</f>
         <v/>
       </c>
-      <c r="J15" s="23" t="n">
+      <c r="J15" s="25" t="n">
         <v>7965</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="26">
         <f>G15*$B$6</f>
         <v/>
       </c>
-      <c r="L15" s="25">
+      <c r="L15" s="27">
         <f>D15*((1+$B$6)^H15-1)*I15</f>
         <v/>
       </c>
-      <c r="M15" s="26">
+      <c r="M15" s="28">
         <f>L15*J15</f>
         <v/>
       </c>
-      <c r="N15" s="27">
+      <c r="N15" s="29">
         <f>M15-K15-L15*$B$7</f>
         <v/>
       </c>
-      <c r="O15" s="28">
+      <c r="O15" s="30">
         <f>K15/L15</f>
         <v/>
       </c>
     </row>
     <row r="16" hidden="1" outlineLevel="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="22" t="n">
         <v>713</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <v>749</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="22" t="n">
         <v>788</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="22" t="n">
         <v>26060</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="22" t="n">
         <v>28666</v>
       </c>
-      <c r="G16" s="20" t="n">
+      <c r="G16" s="22" t="n">
         <v>31533</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="23">
         <f>SLOPE(LN(B16:D16),LN(E16:G16))</f>
         <v/>
       </c>
-      <c r="I16" s="22">
+      <c r="I16" s="24">
         <f>120/1516</f>
         <v/>
       </c>
-      <c r="J16" s="23" t="n">
+      <c r="J16" s="25" t="n">
         <v>7590</v>
       </c>
-      <c r="K16" s="24">
+      <c r="K16" s="26">
         <f>G16*$B$6</f>
         <v/>
       </c>
-      <c r="L16" s="25">
+      <c r="L16" s="27">
         <f>D16*((1+$B$6)^H16-1)*I16</f>
         <v/>
       </c>
-      <c r="M16" s="26">
+      <c r="M16" s="28">
         <f>L16*J16</f>
         <v/>
       </c>
-      <c r="N16" s="27">
+      <c r="N16" s="29">
         <f>M16-K16-L16*$B$7</f>
         <v/>
       </c>
-      <c r="O16" s="28">
+      <c r="O16" s="30">
         <f>K16/L16</f>
         <v/>
       </c>
     </row>
     <row r="17" hidden="1" outlineLevel="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="22" t="n">
         <v>1158</v>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="22" t="n">
         <v>1210</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="22" t="n">
         <v>1265</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="22" t="n">
         <v>56438</v>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="22" t="n">
         <v>62082</v>
       </c>
-      <c r="G17" s="20" t="n">
+      <c r="G17" s="22" t="n">
         <v>68291</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="23">
         <f>SLOPE(LN(B17:D17),LN(E17:G17))</f>
         <v/>
       </c>
-      <c r="I17" s="22">
+      <c r="I17" s="24">
         <f>156/1976</f>
         <v/>
       </c>
-      <c r="J17" s="23" t="n">
+      <c r="J17" s="25" t="n">
         <v>8490</v>
       </c>
-      <c r="K17" s="24">
+      <c r="K17" s="26">
         <f>G17*$B$6</f>
         <v/>
       </c>
-      <c r="L17" s="25">
+      <c r="L17" s="27">
         <f>D17*((1+$B$6)^H17-1)*I17</f>
         <v/>
       </c>
-      <c r="M17" s="26">
+      <c r="M17" s="28">
         <f>L17*J17</f>
         <v/>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="29">
         <f>M17-K17-L17*$B$7</f>
         <v/>
       </c>
-      <c r="O17" s="28">
+      <c r="O17" s="30">
         <f>K17/L17</f>
         <v/>
       </c>
@@ -1244,207 +1286,227 @@
           <t>Iscom</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="13" t="n"/>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="B18" s="13">
+        <f>SUM(B19:B21)</f>
+        <v/>
+      </c>
+      <c r="C18" s="13">
+        <f>SUM(C19:C21)</f>
+        <v/>
+      </c>
+      <c r="D18" s="13">
+        <f>SUM(D19:D21)</f>
+        <v/>
+      </c>
+      <c r="E18" s="14">
+        <f>SUM(E19:E21)</f>
+        <v/>
+      </c>
+      <c r="F18" s="14">
+        <f>SUM(F19:F21)</f>
+        <v/>
+      </c>
+      <c r="G18" s="14">
+        <f>SUM(G19:G21)</f>
+        <v/>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="15">
+      <c r="I18" s="16" t="n">
+        <v>0.07930549038010323</v>
+      </c>
+      <c r="J18" s="17">
         <f>M18/L18</f>
         <v/>
       </c>
-      <c r="K18" s="16">
+      <c r="K18" s="18">
         <f>SUM(K19:K21)</f>
         <v/>
       </c>
-      <c r="L18" s="17">
+      <c r="L18" s="19">
         <f>SUM(L19:L21)</f>
         <v/>
       </c>
-      <c r="M18" s="16">
+      <c r="M18" s="18">
         <f>SUM(M19:M21)</f>
         <v/>
       </c>
-      <c r="N18" s="16">
+      <c r="N18" s="18">
         <f>SUM(N19:N21)</f>
         <v/>
       </c>
-      <c r="O18" s="18">
+      <c r="O18" s="20">
         <f>K18/L18</f>
         <v/>
       </c>
     </row>
     <row r="19" hidden="1" outlineLevel="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="22" t="n">
         <v>571</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="22" t="n">
         <v>600</v>
       </c>
-      <c r="D19" s="20" t="n">
+      <c r="D19" s="22" t="n">
         <v>630</v>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="22" t="n">
         <v>20843</v>
       </c>
-      <c r="F19" s="20" t="n">
+      <c r="F19" s="22" t="n">
         <v>22927</v>
       </c>
-      <c r="G19" s="20" t="n">
+      <c r="G19" s="22" t="n">
         <v>25220</v>
       </c>
-      <c r="H19" s="21">
+      <c r="H19" s="23">
         <f>SLOPE(LN(B19:D19),LN(E19:G19))</f>
         <v/>
       </c>
-      <c r="I19" s="22">
+      <c r="I19" s="24">
         <f>100/1260</f>
         <v/>
       </c>
-      <c r="J19" s="23" t="n">
+      <c r="J19" s="25" t="n">
         <v>7440</v>
       </c>
-      <c r="K19" s="24">
+      <c r="K19" s="26">
         <f>G19*$B$6</f>
         <v/>
       </c>
-      <c r="L19" s="25">
+      <c r="L19" s="27">
         <f>D19*((1+$B$6)^H19-1)*I19</f>
         <v/>
       </c>
-      <c r="M19" s="26">
+      <c r="M19" s="28">
         <f>L19*J19</f>
         <v/>
       </c>
-      <c r="N19" s="27">
+      <c r="N19" s="29">
         <f>M19-K19-L19*$B$7</f>
         <v/>
       </c>
-      <c r="O19" s="28">
+      <c r="O19" s="30">
         <f>K19/L19</f>
         <v/>
       </c>
     </row>
     <row r="20" hidden="1" outlineLevel="1">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="22" t="n">
         <v>1035</v>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="22" t="n">
         <v>1080</v>
       </c>
-      <c r="D20" s="20" t="n">
+      <c r="D20" s="22" t="n">
         <v>1126</v>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="22" t="n">
         <v>50248</v>
       </c>
-      <c r="F20" s="20" t="n">
+      <c r="F20" s="22" t="n">
         <v>55272</v>
       </c>
-      <c r="G20" s="20" t="n">
+      <c r="G20" s="22" t="n">
         <v>60800</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="23">
         <f>SLOPE(LN(B20:D20),LN(E20:G20))</f>
         <v/>
       </c>
-      <c r="I20" s="22">
+      <c r="I20" s="24">
         <f>144/1816</f>
         <v/>
       </c>
-      <c r="J20" s="23" t="n">
+      <c r="J20" s="25" t="n">
         <v>8490</v>
       </c>
-      <c r="K20" s="24">
+      <c r="K20" s="26">
         <f>G20*$B$6</f>
         <v/>
       </c>
-      <c r="L20" s="25">
+      <c r="L20" s="27">
         <f>D20*((1+$B$6)^H20-1)*I20</f>
         <v/>
       </c>
-      <c r="M20" s="26">
+      <c r="M20" s="28">
         <f>L20*J20</f>
         <v/>
       </c>
-      <c r="N20" s="27">
+      <c r="N20" s="29">
         <f>M20-K20-L20*$B$7</f>
         <v/>
       </c>
-      <c r="O20" s="28">
+      <c r="O20" s="30">
         <f>K20/L20</f>
         <v/>
       </c>
     </row>
     <row r="21" hidden="1" outlineLevel="1">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="B21" s="20" t="n">
+      <c r="B21" s="22" t="n">
         <v>526</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="22" t="n">
         <v>553</v>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="22" t="n">
         <v>581</v>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="22" t="n">
         <v>18251</v>
       </c>
-      <c r="F21" s="20" t="n">
+      <c r="F21" s="22" t="n">
         <v>20076</v>
       </c>
-      <c r="G21" s="20" t="n">
+      <c r="G21" s="22" t="n">
         <v>22083</v>
       </c>
-      <c r="H21" s="21">
+      <c r="H21" s="23">
         <f>SLOPE(LN(B21:D21),LN(E21:G21))</f>
         <v/>
       </c>
-      <c r="I21" s="22">
+      <c r="I21" s="24">
         <f>94/1186</f>
         <v/>
       </c>
-      <c r="J21" s="23" t="n">
+      <c r="J21" s="25" t="n">
         <v>7290</v>
       </c>
-      <c r="K21" s="24">
+      <c r="K21" s="26">
         <f>G21*$B$6</f>
         <v/>
       </c>
-      <c r="L21" s="25">
+      <c r="L21" s="27">
         <f>D21*((1+$B$6)^H21-1)*I21</f>
         <v/>
       </c>
-      <c r="M21" s="26">
+      <c r="M21" s="28">
         <f>L21*J21</f>
         <v/>
       </c>
-      <c r="N21" s="27">
+      <c r="N21" s="29">
         <f>M21-K21-L21*$B$7</f>
         <v/>
       </c>
-      <c r="O21" s="28">
+      <c r="O21" s="30">
         <f>K21/L21</f>
         <v/>
       </c>
@@ -1455,207 +1517,227 @@
           <t>Ipac</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="B22" s="13">
+        <f>SUM(B23:B25)</f>
+        <v/>
+      </c>
+      <c r="C22" s="13">
+        <f>SUM(C23:C25)</f>
+        <v/>
+      </c>
+      <c r="D22" s="13">
+        <f>SUM(D23:D25)</f>
+        <v/>
+      </c>
+      <c r="E22" s="14">
+        <f>SUM(E23:E25)</f>
+        <v/>
+      </c>
+      <c r="F22" s="14">
+        <f>SUM(F23:F25)</f>
+        <v/>
+      </c>
+      <c r="G22" s="14">
+        <f>SUM(G23:G25)</f>
+        <v/>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I22" s="13" t="n"/>
-      <c r="J22" s="15">
+      <c r="I22" s="16" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="J22" s="17">
         <f>M22/L22</f>
         <v/>
       </c>
-      <c r="K22" s="16">
+      <c r="K22" s="18">
         <f>SUM(K23:K25)</f>
         <v/>
       </c>
-      <c r="L22" s="17">
+      <c r="L22" s="19">
         <f>SUM(L23:L25)</f>
         <v/>
       </c>
-      <c r="M22" s="16">
+      <c r="M22" s="18">
         <f>SUM(M23:M25)</f>
         <v/>
       </c>
-      <c r="N22" s="16">
+      <c r="N22" s="18">
         <f>SUM(N23:N25)</f>
         <v/>
       </c>
-      <c r="O22" s="18">
+      <c r="O22" s="20">
         <f>K22/L22</f>
         <v/>
       </c>
     </row>
     <row r="23" hidden="1" outlineLevel="1">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Montpellier</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="22" t="n">
         <v>377</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="22" t="n">
         <v>399</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="22" t="n">
         <v>422</v>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E23" s="22" t="n">
         <v>12543</v>
       </c>
-      <c r="F23" s="20" t="n">
+      <c r="F23" s="22" t="n">
         <v>13798</v>
       </c>
-      <c r="G23" s="20" t="n">
+      <c r="G23" s="22" t="n">
         <v>15178</v>
       </c>
-      <c r="H23" s="21">
+      <c r="H23" s="23">
         <f>SLOPE(LN(B23:D23),LN(E23:G23))</f>
         <v/>
       </c>
-      <c r="I23" s="22">
+      <c r="I23" s="24">
         <f>40/680</f>
         <v/>
       </c>
-      <c r="J23" s="23" t="n">
+      <c r="J23" s="25" t="n">
         <v>6740</v>
       </c>
-      <c r="K23" s="24">
+      <c r="K23" s="26">
         <f>G23*$B$6</f>
         <v/>
       </c>
-      <c r="L23" s="25">
+      <c r="L23" s="27">
         <f>D23*((1+$B$6)^H23-1)*I23</f>
         <v/>
       </c>
-      <c r="M23" s="26">
+      <c r="M23" s="28">
         <f>L23*J23</f>
         <v/>
       </c>
-      <c r="N23" s="27">
+      <c r="N23" s="29">
         <f>M23-K23-L23*$B$7</f>
         <v/>
       </c>
-      <c r="O23" s="28">
+      <c r="O23" s="30">
         <f>K23/L23</f>
         <v/>
       </c>
     </row>
     <row r="24" hidden="1" outlineLevel="1">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="22" t="n">
         <v>489</v>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="22" t="n">
         <v>516</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="22" t="n">
         <v>544</v>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="22" t="n">
         <v>17983</v>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="22" t="n">
         <v>19782</v>
       </c>
-      <c r="G24" s="20" t="n">
+      <c r="G24" s="22" t="n">
         <v>21760</v>
       </c>
-      <c r="H24" s="21">
+      <c r="H24" s="23">
         <f>SLOPE(LN(B24:D24),LN(E24:G24))</f>
         <v/>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="24">
         <f>50/850</f>
         <v/>
       </c>
-      <c r="J24" s="23" t="n">
+      <c r="J24" s="25" t="n">
         <v>7090</v>
       </c>
-      <c r="K24" s="24">
+      <c r="K24" s="26">
         <f>G24*$B$6</f>
         <v/>
       </c>
-      <c r="L24" s="25">
+      <c r="L24" s="27">
         <f>D24*((1+$B$6)^H24-1)*I24</f>
         <v/>
       </c>
-      <c r="M24" s="26">
+      <c r="M24" s="28">
         <f>L24*J24</f>
         <v/>
       </c>
-      <c r="N24" s="27">
+      <c r="N24" s="29">
         <f>M24-K24-L24*$B$7</f>
         <v/>
       </c>
-      <c r="O24" s="28">
+      <c r="O24" s="30">
         <f>K24/L24</f>
         <v/>
       </c>
     </row>
     <row r="25" hidden="1" outlineLevel="1">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n">
+      <c r="B25" s="22" t="n">
         <v>371</v>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="22" t="n">
         <v>392</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="22" t="n">
         <v>415</v>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E25" s="22" t="n">
         <v>12341</v>
       </c>
-      <c r="F25" s="20" t="n">
+      <c r="F25" s="22" t="n">
         <v>13575</v>
       </c>
-      <c r="G25" s="20" t="n">
+      <c r="G25" s="22" t="n">
         <v>14933</v>
       </c>
-      <c r="H25" s="21">
+      <c r="H25" s="23">
         <f>SLOPE(LN(B25:D25),LN(E25:G25))</f>
         <v/>
       </c>
-      <c r="I25" s="22">
+      <c r="I25" s="24">
         <f>40/680</f>
         <v/>
       </c>
-      <c r="J25" s="23" t="n">
+      <c r="J25" s="25" t="n">
         <v>6740</v>
       </c>
-      <c r="K25" s="24">
+      <c r="K25" s="26">
         <f>G25*$B$6</f>
         <v/>
       </c>
-      <c r="L25" s="25">
+      <c r="L25" s="27">
         <f>D25*((1+$B$6)^H25-1)*I25</f>
         <v/>
       </c>
-      <c r="M25" s="26">
+      <c r="M25" s="28">
         <f>L25*J25</f>
         <v/>
       </c>
-      <c r="N25" s="27">
+      <c r="N25" s="29">
         <f>M25-K25-L25*$B$7</f>
         <v/>
       </c>
-      <c r="O25" s="28">
+      <c r="O25" s="30">
         <f>K25/L25</f>
         <v/>
       </c>
@@ -1666,151 +1748,171 @@
           <t>Pigier</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="13" t="n"/>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="B26" s="13">
+        <f>SUM(B27:B28)</f>
+        <v/>
+      </c>
+      <c r="C26" s="13">
+        <f>SUM(C27:C28)</f>
+        <v/>
+      </c>
+      <c r="D26" s="13">
+        <f>SUM(D27:D28)</f>
+        <v/>
+      </c>
+      <c r="E26" s="14">
+        <f>SUM(E27:E28)</f>
+        <v/>
+      </c>
+      <c r="F26" s="14">
+        <f>SUM(F27:F28)</f>
+        <v/>
+      </c>
+      <c r="G26" s="14">
+        <f>SUM(G27:G28)</f>
+        <v/>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I26" s="13" t="n"/>
-      <c r="J26" s="15">
+      <c r="I26" s="16" t="n">
+        <v>0.05857142857142857</v>
+      </c>
+      <c r="J26" s="17">
         <f>M26/L26</f>
         <v/>
       </c>
-      <c r="K26" s="16">
+      <c r="K26" s="18">
         <f>SUM(K27:K28)</f>
         <v/>
       </c>
-      <c r="L26" s="17">
+      <c r="L26" s="19">
         <f>SUM(L27:L28)</f>
         <v/>
       </c>
-      <c r="M26" s="16">
+      <c r="M26" s="18">
         <f>SUM(M27:M28)</f>
         <v/>
       </c>
-      <c r="N26" s="16">
+      <c r="N26" s="18">
         <f>SUM(N27:N28)</f>
         <v/>
       </c>
-      <c r="O26" s="18">
+      <c r="O26" s="20">
         <f>K26/L26</f>
         <v/>
       </c>
     </row>
     <row r="27" hidden="1" outlineLevel="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n">
+      <c r="B27" s="22" t="n">
         <v>528</v>
       </c>
-      <c r="C27" s="20" t="n">
+      <c r="C27" s="22" t="n">
         <v>552</v>
       </c>
-      <c r="D27" s="20" t="n">
+      <c r="D27" s="22" t="n">
         <v>578</v>
       </c>
-      <c r="E27" s="20" t="n">
+      <c r="E27" s="22" t="n">
         <v>18155</v>
       </c>
-      <c r="F27" s="20" t="n">
+      <c r="F27" s="22" t="n">
         <v>19971</v>
       </c>
-      <c r="G27" s="20" t="n">
+      <c r="G27" s="22" t="n">
         <v>21968</v>
       </c>
-      <c r="H27" s="21">
+      <c r="H27" s="23">
         <f>SLOPE(LN(B27:D27),LN(E27:G27))</f>
         <v/>
       </c>
-      <c r="I27" s="22">
+      <c r="I27" s="24">
         <f>72/1230</f>
         <v/>
       </c>
-      <c r="J27" s="23" t="n">
+      <c r="J27" s="25" t="n">
         <v>6395</v>
       </c>
-      <c r="K27" s="24">
+      <c r="K27" s="26">
         <f>G27*$B$6</f>
         <v/>
       </c>
-      <c r="L27" s="25">
+      <c r="L27" s="27">
         <f>D27*((1+$B$6)^H27-1)*I27</f>
         <v/>
       </c>
-      <c r="M27" s="26">
+      <c r="M27" s="28">
         <f>L27*J27</f>
         <v/>
       </c>
-      <c r="N27" s="27">
+      <c r="N27" s="29">
         <f>M27-K27-L27*$B$7</f>
         <v/>
       </c>
-      <c r="O27" s="28">
+      <c r="O27" s="30">
         <f>K27/L27</f>
         <v/>
       </c>
     </row>
     <row r="28" hidden="1" outlineLevel="1">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n">
+      <c r="B28" s="22" t="n">
         <v>765</v>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C28" s="22" t="n">
         <v>798</v>
       </c>
-      <c r="D28" s="20" t="n">
+      <c r="D28" s="22" t="n">
         <v>832</v>
       </c>
-      <c r="E28" s="20" t="n">
+      <c r="E28" s="22" t="n">
         <v>30258</v>
       </c>
-      <c r="F28" s="20" t="n">
+      <c r="F28" s="22" t="n">
         <v>33284</v>
       </c>
-      <c r="G28" s="20" t="n">
+      <c r="G28" s="22" t="n">
         <v>36612</v>
       </c>
-      <c r="H28" s="21">
+      <c r="H28" s="23">
         <f>SLOPE(LN(B28:D28),LN(E28:G28))</f>
         <v/>
       </c>
-      <c r="I28" s="22">
+      <c r="I28" s="24">
         <f>92/1570</f>
         <v/>
       </c>
-      <c r="J28" s="23" t="n">
+      <c r="J28" s="25" t="n">
         <v>6915</v>
       </c>
-      <c r="K28" s="24">
+      <c r="K28" s="26">
         <f>G28*$B$6</f>
         <v/>
       </c>
-      <c r="L28" s="25">
+      <c r="L28" s="27">
         <f>D28*((1+$B$6)^H28-1)*I28</f>
         <v/>
       </c>
-      <c r="M28" s="26">
+      <c r="M28" s="28">
         <f>L28*J28</f>
         <v/>
       </c>
-      <c r="N28" s="27">
+      <c r="N28" s="29">
         <f>M28-K28-L28*$B$7</f>
         <v/>
       </c>
-      <c r="O28" s="28">
+      <c r="O28" s="30">
         <f>K28/L28</f>
         <v/>
       </c>
@@ -1821,196 +1923,240 @@
           <t>Tunon</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="13" t="n"/>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="B29" s="13">
+        <f>SUM(B30:B31)</f>
+        <v/>
+      </c>
+      <c r="C29" s="13">
+        <f>SUM(C30:C31)</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>SUM(D30:D31)</f>
+        <v/>
+      </c>
+      <c r="E29" s="14">
+        <f>SUM(E30:E31)</f>
+        <v/>
+      </c>
+      <c r="F29" s="14">
+        <f>SUM(F30:F31)</f>
+        <v/>
+      </c>
+      <c r="G29" s="14">
+        <f>SUM(G30:G31)</f>
+        <v/>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="15">
+      <c r="I29" s="16" t="n">
+        <v>0.05878378378378379</v>
+      </c>
+      <c r="J29" s="17">
         <f>M29/L29</f>
         <v/>
       </c>
-      <c r="K29" s="16">
+      <c r="K29" s="18">
         <f>SUM(K30:K31)</f>
         <v/>
       </c>
-      <c r="L29" s="17">
+      <c r="L29" s="19">
         <f>SUM(L30:L31)</f>
         <v/>
       </c>
-      <c r="M29" s="16">
+      <c r="M29" s="18">
         <f>SUM(M30:M31)</f>
         <v/>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="18">
         <f>SUM(N30:N31)</f>
         <v/>
       </c>
-      <c r="O29" s="18">
+      <c r="O29" s="20">
         <f>K29/L29</f>
         <v/>
       </c>
     </row>
     <row r="30" hidden="1" outlineLevel="1">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="B30" s="20" t="n">
+      <c r="B30" s="22" t="n">
         <v>392</v>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="22" t="n">
         <v>410</v>
       </c>
-      <c r="D30" s="20" t="n">
+      <c r="D30" s="22" t="n">
         <v>428</v>
       </c>
-      <c r="E30" s="20" t="n">
+      <c r="E30" s="22" t="n">
         <v>15578</v>
       </c>
-      <c r="F30" s="20" t="n">
+      <c r="F30" s="22" t="n">
         <v>17136</v>
       </c>
-      <c r="G30" s="20" t="n">
+      <c r="G30" s="22" t="n">
         <v>18850</v>
       </c>
-      <c r="H30" s="21">
+      <c r="H30" s="23">
         <f>SLOPE(LN(B30:D30),LN(E30:G30))</f>
         <v/>
       </c>
-      <c r="I30" s="22">
+      <c r="I30" s="24">
         <f>40/680</f>
         <v/>
       </c>
-      <c r="J30" s="23" t="n">
+      <c r="J30" s="25" t="n">
         <v>7440</v>
       </c>
-      <c r="K30" s="24">
+      <c r="K30" s="26">
         <f>G30*$B$6</f>
         <v/>
       </c>
-      <c r="L30" s="25">
+      <c r="L30" s="27">
         <f>D30*((1+$B$6)^H30-1)*I30</f>
         <v/>
       </c>
-      <c r="M30" s="26">
+      <c r="M30" s="28">
         <f>L30*J30</f>
         <v/>
       </c>
-      <c r="N30" s="27">
+      <c r="N30" s="29">
         <f>M30-K30-L30*$B$7</f>
         <v/>
       </c>
-      <c r="O30" s="28">
+      <c r="O30" s="30">
         <f>K30/L30</f>
         <v/>
       </c>
     </row>
     <row r="31" hidden="1" outlineLevel="1">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="B31" s="20" t="n">
+      <c r="B31" s="22" t="n">
         <v>517</v>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="22" t="n">
         <v>538</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="22" t="n">
         <v>560</v>
       </c>
-      <c r="E31" s="20" t="n">
+      <c r="E31" s="22" t="n">
         <v>24992</v>
       </c>
-      <c r="F31" s="20" t="n">
+      <c r="F31" s="22" t="n">
         <v>27491</v>
       </c>
-      <c r="G31" s="20" t="n">
+      <c r="G31" s="22" t="n">
         <v>30240</v>
       </c>
-      <c r="H31" s="21">
+      <c r="H31" s="23">
         <f>SLOPE(LN(B31:D31),LN(E31:G31))</f>
         <v/>
       </c>
-      <c r="I31" s="22">
+      <c r="I31" s="24">
         <f>47/800</f>
         <v/>
       </c>
-      <c r="J31" s="23" t="n">
+      <c r="J31" s="25" t="n">
         <v>7930</v>
       </c>
-      <c r="K31" s="24">
+      <c r="K31" s="26">
         <f>G31*$B$6</f>
         <v/>
       </c>
-      <c r="L31" s="25">
+      <c r="L31" s="27">
         <f>D31*((1+$B$6)^H31-1)*I31</f>
         <v/>
       </c>
-      <c r="M31" s="26">
+      <c r="M31" s="28">
         <f>L31*J31</f>
         <v/>
       </c>
-      <c r="N31" s="27">
+      <c r="N31" s="29">
         <f>M31-K31-L31*$B$7</f>
         <v/>
       </c>
-      <c r="O31" s="28">
+      <c r="O31" s="30">
         <f>K31/L31</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="29" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>GROUPE</t>
         </is>
       </c>
-      <c r="B32" s="30" t="n"/>
-      <c r="C32" s="30" t="n"/>
-      <c r="D32" s="30" t="n"/>
-      <c r="E32" s="30" t="n"/>
-      <c r="F32" s="30" t="n"/>
-      <c r="G32" s="30" t="n"/>
-      <c r="H32" s="30" t="n"/>
-      <c r="I32" s="30" t="n"/>
-      <c r="J32" s="31">
+      <c r="B32" s="32">
+        <f>B14+B15+B16+B17+B19+B20+B21+B23+B24+B25+B27+B28+B30+B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="32">
+        <f>C14+C15+C16+C17+C19+C20+C21+C23+C24+C25+C27+C28+C30+C31</f>
+        <v/>
+      </c>
+      <c r="D32" s="32">
+        <f>D14+D15+D16+D17+D19+D20+D21+D23+D24+D25+D27+D28+D30+D31</f>
+        <v/>
+      </c>
+      <c r="E32" s="33">
+        <f>E14+E15+E16+E17+E19+E20+E21+E23+E24+E25+E27+E28+E30+E31</f>
+        <v/>
+      </c>
+      <c r="F32" s="33">
+        <f>F14+F15+F16+F17+F19+F20+F21+F23+F24+F25+F27+F28+F30+F31</f>
+        <v/>
+      </c>
+      <c r="G32" s="33">
+        <f>G14+G15+G16+G17+G19+G20+G21+G23+G24+G25+G27+G28+G30+G31</f>
+        <v/>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="35" t="n">
+        <v>0.07147010932775064</v>
+      </c>
+      <c r="J32" s="33">
         <f>M32/L32</f>
         <v/>
       </c>
-      <c r="K32" s="32">
+      <c r="K32" s="36">
         <f>K14+K15+K16+K17+K19+K20+K21+K23+K24+K25+K27+K28+K30+K31</f>
         <v/>
       </c>
-      <c r="L32" s="33">
+      <c r="L32" s="37">
         <f>L14+L15+L16+L17+L19+L20+L21+L23+L24+L25+L27+L28+L30+L31</f>
         <v/>
       </c>
-      <c r="M32" s="32">
+      <c r="M32" s="36">
         <f>M14+M15+M16+M17+M19+M20+M21+M23+M24+M25+M27+M28+M30+M31</f>
         <v/>
       </c>
-      <c r="N32" s="32">
+      <c r="N32" s="36">
         <f>N14+N15+N16+N17+N19+N20+N21+N23+N24+N25+N27+N28+N30+N31</f>
         <v/>
       </c>
-      <c r="O32" s="34">
+      <c r="O32" s="38">
         <f>K32/L32</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="35" t="inlineStr">
+      <c r="A34" s="39" t="inlineStr">
         <is>
           <t>Déplie une marque (le +) : chaque campus a SA vraie élasticité (=SLOPE, comme le moteur). Le CAC marginal marque = Σbudget ÷ Σinscrits (agrégat réel).</t>
         </is>
@@ -2024,7 +2170,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="36" t="inlineStr">
+      <c r="A38" s="40" t="inlineStr">
         <is>
           <t>Payants : élasticité 24→25 × budget26. Organiques : leur tendance 24→25. × conversion 2025 → inscrits. Rien de 2026 en entrée.</t>
         </is>
@@ -2123,947 +2269,947 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="37" t="inlineStr">
+      <c r="A41" s="41" t="inlineStr">
         <is>
           <t>Ipac Montpellier</t>
         </is>
       </c>
-      <c r="B41" s="38" t="n">
+      <c r="B41" s="42" t="n">
         <v>377</v>
       </c>
-      <c r="C41" s="38" t="n">
+      <c r="C41" s="42" t="n">
         <v>399</v>
       </c>
-      <c r="D41" s="38" t="n">
+      <c r="D41" s="42" t="n">
         <v>12543</v>
       </c>
-      <c r="E41" s="38" t="n">
+      <c r="E41" s="42" t="n">
         <v>13798</v>
       </c>
-      <c r="F41" s="38" t="n">
+      <c r="F41" s="42" t="n">
         <v>15178</v>
       </c>
-      <c r="G41" s="39">
+      <c r="G41" s="43">
         <f>LN(C41/B41)/LN(E41/D41)</f>
         <v/>
       </c>
-      <c r="H41" s="40">
+      <c r="H41" s="44">
         <f>C41*(F41/E41)^G41</f>
         <v/>
       </c>
-      <c r="I41" s="38" t="n">
+      <c r="I41" s="42" t="n">
         <v>217</v>
       </c>
-      <c r="J41" s="38" t="n">
+      <c r="J41" s="42" t="n">
         <v>237</v>
       </c>
-      <c r="K41" s="40">
+      <c r="K41" s="44">
         <f>J41*(J41/I41)</f>
         <v/>
       </c>
-      <c r="L41" s="41">
+      <c r="L41" s="45">
         <f>H41+K41</f>
         <v/>
       </c>
-      <c r="M41" s="38" t="n">
+      <c r="M41" s="42" t="n">
         <v>642</v>
       </c>
-      <c r="N41" s="38" t="n">
+      <c r="N41" s="42" t="n">
         <v>38</v>
       </c>
-      <c r="O41" s="42">
+      <c r="O41" s="46">
         <f>N41/M41</f>
         <v/>
       </c>
-      <c r="P41" s="41">
+      <c r="P41" s="45">
         <f>L41*O41</f>
         <v/>
       </c>
-      <c r="Q41" s="43" t="n">
+      <c r="Q41" s="47" t="n">
         <v>40</v>
       </c>
-      <c r="R41" s="44">
+      <c r="R41" s="48">
         <f>P41/Q41-1</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="37" t="inlineStr">
+      <c r="A42" s="41" t="inlineStr">
         <is>
           <t>Ipac Nantes</t>
         </is>
       </c>
-      <c r="B42" s="38" t="n">
+      <c r="B42" s="42" t="n">
         <v>489</v>
       </c>
-      <c r="C42" s="38" t="n">
+      <c r="C42" s="42" t="n">
         <v>516</v>
       </c>
-      <c r="D42" s="38" t="n">
+      <c r="D42" s="42" t="n">
         <v>17983</v>
       </c>
-      <c r="E42" s="38" t="n">
+      <c r="E42" s="42" t="n">
         <v>19782</v>
       </c>
-      <c r="F42" s="38" t="n">
+      <c r="F42" s="42" t="n">
         <v>21760</v>
       </c>
-      <c r="G42" s="39">
+      <c r="G42" s="43">
         <f>LN(C42/B42)/LN(E42/D42)</f>
         <v/>
       </c>
-      <c r="H42" s="40">
+      <c r="H42" s="44">
         <f>C42*(F42/E42)^G42</f>
         <v/>
       </c>
-      <c r="I42" s="38" t="n">
+      <c r="I42" s="42" t="n">
         <v>258</v>
       </c>
-      <c r="J42" s="38" t="n">
+      <c r="J42" s="42" t="n">
         <v>281</v>
       </c>
-      <c r="K42" s="40">
+      <c r="K42" s="44">
         <f>J42*(J42/I42)</f>
         <v/>
       </c>
-      <c r="L42" s="41">
+      <c r="L42" s="45">
         <f>H42+K42</f>
         <v/>
       </c>
-      <c r="M42" s="38" t="n">
+      <c r="M42" s="42" t="n">
         <v>802</v>
       </c>
-      <c r="N42" s="38" t="n">
+      <c r="N42" s="42" t="n">
         <v>47</v>
       </c>
-      <c r="O42" s="42">
+      <c r="O42" s="46">
         <f>N42/M42</f>
         <v/>
       </c>
-      <c r="P42" s="41">
+      <c r="P42" s="45">
         <f>L42*O42</f>
         <v/>
       </c>
-      <c r="Q42" s="43" t="n">
+      <c r="Q42" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="R42" s="44">
+      <c r="R42" s="48">
         <f>P42/Q42-1</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="37" t="inlineStr">
+      <c r="A43" s="41" t="inlineStr">
         <is>
           <t>Ipac Rennes</t>
         </is>
       </c>
-      <c r="B43" s="38" t="n">
+      <c r="B43" s="42" t="n">
         <v>371</v>
       </c>
-      <c r="C43" s="38" t="n">
+      <c r="C43" s="42" t="n">
         <v>392</v>
       </c>
-      <c r="D43" s="38" t="n">
+      <c r="D43" s="42" t="n">
         <v>12341</v>
       </c>
-      <c r="E43" s="38" t="n">
+      <c r="E43" s="42" t="n">
         <v>13575</v>
       </c>
-      <c r="F43" s="38" t="n">
+      <c r="F43" s="42" t="n">
         <v>14933</v>
       </c>
-      <c r="G43" s="39">
+      <c r="G43" s="43">
         <f>LN(C43/B43)/LN(E43/D43)</f>
         <v/>
       </c>
-      <c r="H43" s="40">
+      <c r="H43" s="44">
         <f>C43*(F43/E43)^G43</f>
         <v/>
       </c>
-      <c r="I43" s="38" t="n">
+      <c r="I43" s="42" t="n">
         <v>223</v>
       </c>
-      <c r="J43" s="38" t="n">
+      <c r="J43" s="42" t="n">
         <v>243</v>
       </c>
-      <c r="K43" s="40">
+      <c r="K43" s="44">
         <f>J43*(J43/I43)</f>
         <v/>
       </c>
-      <c r="L43" s="41">
+      <c r="L43" s="45">
         <f>H43+K43</f>
         <v/>
       </c>
-      <c r="M43" s="38" t="n">
+      <c r="M43" s="42" t="n">
         <v>642</v>
       </c>
-      <c r="N43" s="38" t="n">
+      <c r="N43" s="42" t="n">
         <v>38</v>
       </c>
-      <c r="O43" s="42">
+      <c r="O43" s="46">
         <f>N43/M43</f>
         <v/>
       </c>
-      <c r="P43" s="41">
+      <c r="P43" s="45">
         <f>L43*O43</f>
         <v/>
       </c>
-      <c r="Q43" s="43" t="n">
+      <c r="Q43" s="47" t="n">
         <v>40</v>
       </c>
-      <c r="R43" s="44">
+      <c r="R43" s="48">
         <f>P43/Q43-1</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="37" t="inlineStr">
+      <c r="A44" s="41" t="inlineStr">
         <is>
           <t>Iscom Lille</t>
         </is>
       </c>
-      <c r="B44" s="38" t="n">
+      <c r="B44" s="42" t="n">
         <v>571</v>
       </c>
-      <c r="C44" s="38" t="n">
+      <c r="C44" s="42" t="n">
         <v>600</v>
       </c>
-      <c r="D44" s="38" t="n">
+      <c r="D44" s="42" t="n">
         <v>20843</v>
       </c>
-      <c r="E44" s="38" t="n">
+      <c r="E44" s="42" t="n">
         <v>22927</v>
       </c>
-      <c r="F44" s="38" t="n">
+      <c r="F44" s="42" t="n">
         <v>25220</v>
       </c>
-      <c r="G44" s="39">
+      <c r="G44" s="43">
         <f>LN(C44/B44)/LN(E44/D44)</f>
         <v/>
       </c>
-      <c r="H44" s="40">
+      <c r="H44" s="44">
         <f>C44*(F44/E44)^G44</f>
         <v/>
       </c>
-      <c r="I44" s="38" t="n">
+      <c r="I44" s="42" t="n">
         <v>594</v>
       </c>
-      <c r="J44" s="38" t="n">
+      <c r="J44" s="42" t="n">
         <v>612</v>
       </c>
-      <c r="K44" s="40">
+      <c r="K44" s="44">
         <f>J44*(J44/I44)</f>
         <v/>
       </c>
-      <c r="L44" s="41">
+      <c r="L44" s="45">
         <f>H44+K44</f>
         <v/>
       </c>
-      <c r="M44" s="38" t="n">
+      <c r="M44" s="42" t="n">
         <v>1190</v>
       </c>
-      <c r="N44" s="38" t="n">
+      <c r="N44" s="42" t="n">
         <v>94</v>
       </c>
-      <c r="O44" s="42">
+      <c r="O44" s="46">
         <f>N44/M44</f>
         <v/>
       </c>
-      <c r="P44" s="41">
+      <c r="P44" s="45">
         <f>L44*O44</f>
         <v/>
       </c>
-      <c r="Q44" s="43" t="n">
+      <c r="Q44" s="47" t="n">
         <v>100</v>
       </c>
-      <c r="R44" s="44">
+      <c r="R44" s="48">
         <f>P44/Q44-1</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="37" t="inlineStr">
+      <c r="A45" s="41" t="inlineStr">
         <is>
           <t>Iscom Paris</t>
         </is>
       </c>
-      <c r="B45" s="38" t="n">
+      <c r="B45" s="42" t="n">
         <v>1035</v>
       </c>
-      <c r="C45" s="38" t="n">
+      <c r="C45" s="42" t="n">
         <v>1080</v>
       </c>
-      <c r="D45" s="38" t="n">
+      <c r="D45" s="42" t="n">
         <v>50248</v>
       </c>
-      <c r="E45" s="38" t="n">
+      <c r="E45" s="42" t="n">
         <v>55272</v>
       </c>
-      <c r="F45" s="38" t="n">
+      <c r="F45" s="42" t="n">
         <v>60800</v>
       </c>
-      <c r="G45" s="39">
+      <c r="G45" s="43">
         <f>LN(C45/B45)/LN(E45/D45)</f>
         <v/>
       </c>
-      <c r="H45" s="40">
+      <c r="H45" s="44">
         <f>C45*(F45/E45)^G45</f>
         <v/>
       </c>
-      <c r="I45" s="38" t="n">
+      <c r="I45" s="42" t="n">
         <v>650</v>
       </c>
-      <c r="J45" s="38" t="n">
+      <c r="J45" s="42" t="n">
         <v>670</v>
       </c>
-      <c r="K45" s="40">
+      <c r="K45" s="44">
         <f>J45*(J45/I45)</f>
         <v/>
       </c>
-      <c r="L45" s="41">
+      <c r="L45" s="45">
         <f>H45+K45</f>
         <v/>
       </c>
-      <c r="M45" s="38" t="n">
+      <c r="M45" s="42" t="n">
         <v>1713</v>
       </c>
-      <c r="N45" s="38" t="n">
+      <c r="N45" s="42" t="n">
         <v>136</v>
       </c>
-      <c r="O45" s="42">
+      <c r="O45" s="46">
         <f>N45/M45</f>
         <v/>
       </c>
-      <c r="P45" s="41">
+      <c r="P45" s="45">
         <f>L45*O45</f>
         <v/>
       </c>
-      <c r="Q45" s="43" t="n">
+      <c r="Q45" s="47" t="n">
         <v>144</v>
       </c>
-      <c r="R45" s="44">
+      <c r="R45" s="48">
         <f>P45/Q45-1</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="37" t="inlineStr">
+      <c r="A46" s="41" t="inlineStr">
         <is>
           <t>Iscom Toulouse</t>
         </is>
       </c>
-      <c r="B46" s="38" t="n">
+      <c r="B46" s="42" t="n">
         <v>526</v>
       </c>
-      <c r="C46" s="38" t="n">
+      <c r="C46" s="42" t="n">
         <v>553</v>
       </c>
-      <c r="D46" s="38" t="n">
+      <c r="D46" s="42" t="n">
         <v>18251</v>
       </c>
-      <c r="E46" s="38" t="n">
+      <c r="E46" s="42" t="n">
         <v>20076</v>
       </c>
-      <c r="F46" s="38" t="n">
+      <c r="F46" s="42" t="n">
         <v>22083</v>
       </c>
-      <c r="G46" s="39">
+      <c r="G46" s="43">
         <f>LN(C46/B46)/LN(E46/D46)</f>
         <v/>
       </c>
-      <c r="H46" s="40">
+      <c r="H46" s="44">
         <f>C46*(F46/E46)^G46</f>
         <v/>
       </c>
-      <c r="I46" s="38" t="n">
+      <c r="I46" s="42" t="n">
         <v>570</v>
       </c>
-      <c r="J46" s="38" t="n">
+      <c r="J46" s="42" t="n">
         <v>587</v>
       </c>
-      <c r="K46" s="40">
+      <c r="K46" s="44">
         <f>J46*(J46/I46)</f>
         <v/>
       </c>
-      <c r="L46" s="41">
+      <c r="L46" s="45">
         <f>H46+K46</f>
         <v/>
       </c>
-      <c r="M46" s="38" t="n">
+      <c r="M46" s="42" t="n">
         <v>1119</v>
       </c>
-      <c r="N46" s="38" t="n">
+      <c r="N46" s="42" t="n">
         <v>88</v>
       </c>
-      <c r="O46" s="42">
+      <c r="O46" s="46">
         <f>N46/M46</f>
         <v/>
       </c>
-      <c r="P46" s="41">
+      <c r="P46" s="45">
         <f>L46*O46</f>
         <v/>
       </c>
-      <c r="Q46" s="43" t="n">
+      <c r="Q46" s="47" t="n">
         <v>94</v>
       </c>
-      <c r="R46" s="44">
+      <c r="R46" s="48">
         <f>P46/Q46-1</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="37" t="inlineStr">
+      <c r="A47" s="41" t="inlineStr">
         <is>
           <t>MBway Bordeaux</t>
         </is>
       </c>
-      <c r="B47" s="38" t="n">
+      <c r="B47" s="42" t="n">
         <v>592</v>
       </c>
-      <c r="C47" s="38" t="n">
+      <c r="C47" s="42" t="n">
         <v>623</v>
       </c>
-      <c r="D47" s="38" t="n">
+      <c r="D47" s="42" t="n">
         <v>20597</v>
       </c>
-      <c r="E47" s="38" t="n">
+      <c r="E47" s="42" t="n">
         <v>22657</v>
       </c>
-      <c r="F47" s="38" t="n">
+      <c r="F47" s="42" t="n">
         <v>24923</v>
       </c>
-      <c r="G47" s="39">
+      <c r="G47" s="43">
         <f>LN(C47/B47)/LN(E47/D47)</f>
         <v/>
       </c>
-      <c r="H47" s="40">
+      <c r="H47" s="44">
         <f>C47*(F47/E47)^G47</f>
         <v/>
       </c>
-      <c r="I47" s="38" t="n">
+      <c r="I47" s="42" t="n">
         <v>550</v>
       </c>
-      <c r="J47" s="38" t="n">
+      <c r="J47" s="42" t="n">
         <v>589</v>
       </c>
-      <c r="K47" s="40">
+      <c r="K47" s="44">
         <f>J47*(J47/I47)</f>
         <v/>
       </c>
-      <c r="L47" s="41">
+      <c r="L47" s="45">
         <f>H47+K47</f>
         <v/>
       </c>
-      <c r="M47" s="38" t="n">
+      <c r="M47" s="42" t="n">
         <v>1213</v>
       </c>
-      <c r="N47" s="38" t="n">
+      <c r="N47" s="42" t="n">
         <v>96</v>
       </c>
-      <c r="O47" s="42">
+      <c r="O47" s="46">
         <f>N47/M47</f>
         <v/>
       </c>
-      <c r="P47" s="41">
+      <c r="P47" s="45">
         <f>L47*O47</f>
         <v/>
       </c>
-      <c r="Q47" s="43" t="n">
+      <c r="Q47" s="47" t="n">
         <v>102</v>
       </c>
-      <c r="R47" s="44">
+      <c r="R47" s="48">
         <f>P47/Q47-1</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="37" t="inlineStr">
+      <c r="A48" s="41" t="inlineStr">
         <is>
           <t>MBway Lyon</t>
         </is>
       </c>
-      <c r="B48" s="38" t="n">
+      <c r="B48" s="42" t="n">
         <v>863</v>
       </c>
-      <c r="C48" s="38" t="n">
+      <c r="C48" s="42" t="n">
         <v>905</v>
       </c>
-      <c r="D48" s="38" t="n">
+      <c r="D48" s="42" t="n">
         <v>34532</v>
       </c>
-      <c r="E48" s="38" t="n">
+      <c r="E48" s="42" t="n">
         <v>37985</v>
       </c>
-      <c r="F48" s="38" t="n">
+      <c r="F48" s="42" t="n">
         <v>41783</v>
       </c>
-      <c r="G48" s="39">
+      <c r="G48" s="43">
         <f>LN(C48/B48)/LN(E48/D48)</f>
         <v/>
       </c>
-      <c r="H48" s="40">
+      <c r="H48" s="44">
         <f>C48*(F48/E48)^G48</f>
         <v/>
       </c>
-      <c r="I48" s="38" t="n">
+      <c r="I48" s="42" t="n">
         <v>626</v>
       </c>
-      <c r="J48" s="38" t="n">
+      <c r="J48" s="42" t="n">
         <v>670</v>
       </c>
-      <c r="K48" s="40">
+      <c r="K48" s="44">
         <f>J48*(J48/I48)</f>
         <v/>
       </c>
-      <c r="L48" s="41">
+      <c r="L48" s="45">
         <f>H48+K48</f>
         <v/>
       </c>
-      <c r="M48" s="38" t="n">
+      <c r="M48" s="42" t="n">
         <v>1572</v>
       </c>
-      <c r="N48" s="38" t="n">
+      <c r="N48" s="42" t="n">
         <v>124</v>
       </c>
-      <c r="O48" s="42">
+      <c r="O48" s="46">
         <f>N48/M48</f>
         <v/>
       </c>
-      <c r="P48" s="41">
+      <c r="P48" s="45">
         <f>L48*O48</f>
         <v/>
       </c>
-      <c r="Q48" s="43" t="n">
+      <c r="Q48" s="47" t="n">
         <v>132</v>
       </c>
-      <c r="R48" s="44">
+      <c r="R48" s="48">
         <f>P48/Q48-1</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="37" t="inlineStr">
+      <c r="A49" s="41" t="inlineStr">
         <is>
           <t>MBway Nantes</t>
         </is>
       </c>
-      <c r="B49" s="38" t="n">
+      <c r="B49" s="42" t="n">
         <v>713</v>
       </c>
-      <c r="C49" s="38" t="n">
+      <c r="C49" s="42" t="n">
         <v>749</v>
       </c>
-      <c r="D49" s="38" t="n">
+      <c r="D49" s="42" t="n">
         <v>26060</v>
       </c>
-      <c r="E49" s="38" t="n">
+      <c r="E49" s="42" t="n">
         <v>28666</v>
       </c>
-      <c r="F49" s="38" t="n">
+      <c r="F49" s="42" t="n">
         <v>31533</v>
       </c>
-      <c r="G49" s="39">
+      <c r="G49" s="43">
         <f>LN(C49/B49)/LN(E49/D49)</f>
         <v/>
       </c>
-      <c r="H49" s="40">
+      <c r="H49" s="44">
         <f>C49*(F49/E49)^G49</f>
         <v/>
       </c>
-      <c r="I49" s="38" t="n">
+      <c r="I49" s="42" t="n">
         <v>636</v>
       </c>
-      <c r="J49" s="38" t="n">
+      <c r="J49" s="42" t="n">
         <v>680</v>
       </c>
-      <c r="K49" s="40">
+      <c r="K49" s="44">
         <f>J49*(J49/I49)</f>
         <v/>
       </c>
-      <c r="L49" s="41">
+      <c r="L49" s="45">
         <f>H49+K49</f>
         <v/>
       </c>
-      <c r="M49" s="38" t="n">
+      <c r="M49" s="42" t="n">
         <v>1430</v>
       </c>
-      <c r="N49" s="38" t="n">
+      <c r="N49" s="42" t="n">
         <v>114</v>
       </c>
-      <c r="O49" s="42">
+      <c r="O49" s="46">
         <f>N49/M49</f>
         <v/>
       </c>
-      <c r="P49" s="41">
+      <c r="P49" s="45">
         <f>L49*O49</f>
         <v/>
       </c>
-      <c r="Q49" s="43" t="n">
+      <c r="Q49" s="47" t="n">
         <v>120</v>
       </c>
-      <c r="R49" s="44">
+      <c r="R49" s="48">
         <f>P49/Q49-1</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="37" t="inlineStr">
+      <c r="A50" s="41" t="inlineStr">
         <is>
           <t>MBway Paris</t>
         </is>
       </c>
-      <c r="B50" s="38" t="n">
+      <c r="B50" s="42" t="n">
         <v>1158</v>
       </c>
-      <c r="C50" s="38" t="n">
+      <c r="C50" s="42" t="n">
         <v>1210</v>
       </c>
-      <c r="D50" s="38" t="n">
+      <c r="D50" s="42" t="n">
         <v>56438</v>
       </c>
-      <c r="E50" s="38" t="n">
+      <c r="E50" s="42" t="n">
         <v>62082</v>
       </c>
-      <c r="F50" s="38" t="n">
+      <c r="F50" s="42" t="n">
         <v>68291</v>
       </c>
-      <c r="G50" s="39">
+      <c r="G50" s="43">
         <f>LN(C50/B50)/LN(E50/D50)</f>
         <v/>
       </c>
-      <c r="H50" s="40">
+      <c r="H50" s="44">
         <f>C50*(F50/E50)^G50</f>
         <v/>
       </c>
-      <c r="I50" s="38" t="n">
+      <c r="I50" s="42" t="n">
         <v>621</v>
       </c>
-      <c r="J50" s="38" t="n">
+      <c r="J50" s="42" t="n">
         <v>665</v>
       </c>
-      <c r="K50" s="40">
+      <c r="K50" s="44">
         <f>J50*(J50/I50)</f>
         <v/>
       </c>
-      <c r="L50" s="41">
+      <c r="L50" s="45">
         <f>H50+K50</f>
         <v/>
       </c>
-      <c r="M50" s="38" t="n">
+      <c r="M50" s="42" t="n">
         <v>1864</v>
       </c>
-      <c r="N50" s="38" t="n">
+      <c r="N50" s="42" t="n">
         <v>148</v>
       </c>
-      <c r="O50" s="42">
+      <c r="O50" s="46">
         <f>N50/M50</f>
         <v/>
       </c>
-      <c r="P50" s="41">
+      <c r="P50" s="45">
         <f>L50*O50</f>
         <v/>
       </c>
-      <c r="Q50" s="43" t="n">
+      <c r="Q50" s="47" t="n">
         <v>156</v>
       </c>
-      <c r="R50" s="44">
+      <c r="R50" s="48">
         <f>P50/Q50-1</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="37" t="inlineStr">
+      <c r="A51" s="41" t="inlineStr">
         <is>
           <t>Pigier Bordeaux</t>
         </is>
       </c>
-      <c r="B51" s="38" t="n">
+      <c r="B51" s="42" t="n">
         <v>528</v>
       </c>
-      <c r="C51" s="38" t="n">
+      <c r="C51" s="42" t="n">
         <v>552</v>
       </c>
-      <c r="D51" s="38" t="n">
+      <c r="D51" s="42" t="n">
         <v>18155</v>
       </c>
-      <c r="E51" s="38" t="n">
+      <c r="E51" s="42" t="n">
         <v>19971</v>
       </c>
-      <c r="F51" s="38" t="n">
+      <c r="F51" s="42" t="n">
         <v>21968</v>
       </c>
-      <c r="G51" s="39">
+      <c r="G51" s="43">
         <f>LN(C51/B51)/LN(E51/D51)</f>
         <v/>
       </c>
-      <c r="H51" s="40">
+      <c r="H51" s="44">
         <f>C51*(F51/E51)^G51</f>
         <v/>
       </c>
-      <c r="I51" s="38" t="n">
+      <c r="I51" s="42" t="n">
         <v>603</v>
       </c>
-      <c r="J51" s="38" t="n">
+      <c r="J51" s="42" t="n">
         <v>627</v>
       </c>
-      <c r="K51" s="40">
+      <c r="K51" s="44">
         <f>J51*(J51/I51)</f>
         <v/>
       </c>
-      <c r="L51" s="41">
+      <c r="L51" s="45">
         <f>H51+K51</f>
         <v/>
       </c>
-      <c r="M51" s="38" t="n">
+      <c r="M51" s="42" t="n">
         <v>1160</v>
       </c>
-      <c r="N51" s="38" t="n">
+      <c r="N51" s="42" t="n">
         <v>68</v>
       </c>
-      <c r="O51" s="42">
+      <c r="O51" s="46">
         <f>N51/M51</f>
         <v/>
       </c>
-      <c r="P51" s="41">
+      <c r="P51" s="45">
         <f>L51*O51</f>
         <v/>
       </c>
-      <c r="Q51" s="43" t="n">
+      <c r="Q51" s="47" t="n">
         <v>72</v>
       </c>
-      <c r="R51" s="44">
+      <c r="R51" s="48">
         <f>P51/Q51-1</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="37" t="inlineStr">
+      <c r="A52" s="41" t="inlineStr">
         <is>
           <t>Pigier Lyon</t>
         </is>
       </c>
-      <c r="B52" s="38" t="n">
+      <c r="B52" s="42" t="n">
         <v>765</v>
       </c>
-      <c r="C52" s="38" t="n">
+      <c r="C52" s="42" t="n">
         <v>798</v>
       </c>
-      <c r="D52" s="38" t="n">
+      <c r="D52" s="42" t="n">
         <v>30258</v>
       </c>
-      <c r="E52" s="38" t="n">
+      <c r="E52" s="42" t="n">
         <v>33284</v>
       </c>
-      <c r="F52" s="38" t="n">
+      <c r="F52" s="42" t="n">
         <v>36612</v>
       </c>
-      <c r="G52" s="39">
+      <c r="G52" s="43">
         <f>LN(C52/B52)/LN(E52/D52)</f>
         <v/>
       </c>
-      <c r="H52" s="40">
+      <c r="H52" s="44">
         <f>C52*(F52/E52)^G52</f>
         <v/>
       </c>
-      <c r="I52" s="38" t="n">
+      <c r="I52" s="42" t="n">
         <v>682</v>
       </c>
-      <c r="J52" s="38" t="n">
+      <c r="J52" s="42" t="n">
         <v>710</v>
       </c>
-      <c r="K52" s="40">
+      <c r="K52" s="44">
         <f>J52*(J52/I52)</f>
         <v/>
       </c>
-      <c r="L52" s="41">
+      <c r="L52" s="45">
         <f>H52+K52</f>
         <v/>
       </c>
-      <c r="M52" s="38" t="n">
+      <c r="M52" s="42" t="n">
         <v>1482</v>
       </c>
-      <c r="N52" s="38" t="n">
+      <c r="N52" s="42" t="n">
         <v>86</v>
       </c>
-      <c r="O52" s="42">
+      <c r="O52" s="46">
         <f>N52/M52</f>
         <v/>
       </c>
-      <c r="P52" s="41">
+      <c r="P52" s="45">
         <f>L52*O52</f>
         <v/>
       </c>
-      <c r="Q52" s="43" t="n">
+      <c r="Q52" s="47" t="n">
         <v>92</v>
       </c>
-      <c r="R52" s="44">
+      <c r="R52" s="48">
         <f>P52/Q52-1</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="37" t="inlineStr">
+      <c r="A53" s="41" t="inlineStr">
         <is>
           <t>Tunon Lyon</t>
         </is>
       </c>
-      <c r="B53" s="38" t="n">
+      <c r="B53" s="42" t="n">
         <v>392</v>
       </c>
-      <c r="C53" s="38" t="n">
+      <c r="C53" s="42" t="n">
         <v>410</v>
       </c>
-      <c r="D53" s="38" t="n">
+      <c r="D53" s="42" t="n">
         <v>15578</v>
       </c>
-      <c r="E53" s="38" t="n">
+      <c r="E53" s="42" t="n">
         <v>17136</v>
       </c>
-      <c r="F53" s="38" t="n">
+      <c r="F53" s="42" t="n">
         <v>18850</v>
       </c>
-      <c r="G53" s="39">
+      <c r="G53" s="43">
         <f>LN(C53/B53)/LN(E53/D53)</f>
         <v/>
       </c>
-      <c r="H53" s="40">
+      <c r="H53" s="44">
         <f>C53*(F53/E53)^G53</f>
         <v/>
       </c>
-      <c r="I53" s="38" t="n">
+      <c r="I53" s="42" t="n">
         <v>242</v>
       </c>
-      <c r="J53" s="38" t="n">
+      <c r="J53" s="42" t="n">
         <v>247</v>
       </c>
-      <c r="K53" s="40">
+      <c r="K53" s="44">
         <f>J53*(J53/I53)</f>
         <v/>
       </c>
-      <c r="L53" s="41">
+      <c r="L53" s="45">
         <f>H53+K53</f>
         <v/>
       </c>
-      <c r="M53" s="38" t="n">
+      <c r="M53" s="42" t="n">
         <v>642</v>
       </c>
-      <c r="N53" s="38" t="n">
+      <c r="N53" s="42" t="n">
         <v>38</v>
       </c>
-      <c r="O53" s="42">
+      <c r="O53" s="46">
         <f>N53/M53</f>
         <v/>
       </c>
-      <c r="P53" s="41">
+      <c r="P53" s="45">
         <f>L53*O53</f>
         <v/>
       </c>
-      <c r="Q53" s="43" t="n">
+      <c r="Q53" s="47" t="n">
         <v>40</v>
       </c>
-      <c r="R53" s="44">
+      <c r="R53" s="48">
         <f>P53/Q53-1</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="37" t="inlineStr">
+      <c r="A54" s="41" t="inlineStr">
         <is>
           <t>Tunon Paris</t>
         </is>
       </c>
-      <c r="B54" s="38" t="n">
+      <c r="B54" s="42" t="n">
         <v>517</v>
       </c>
-      <c r="C54" s="38" t="n">
+      <c r="C54" s="42" t="n">
         <v>538</v>
       </c>
-      <c r="D54" s="38" t="n">
+      <c r="D54" s="42" t="n">
         <v>24992</v>
       </c>
-      <c r="E54" s="38" t="n">
+      <c r="E54" s="42" t="n">
         <v>27491</v>
       </c>
-      <c r="F54" s="38" t="n">
+      <c r="F54" s="42" t="n">
         <v>30240</v>
       </c>
-      <c r="G54" s="39">
+      <c r="G54" s="43">
         <f>LN(C54/B54)/LN(E54/D54)</f>
         <v/>
       </c>
-      <c r="H54" s="40">
+      <c r="H54" s="44">
         <f>C54*(F54/E54)^G54</f>
         <v/>
       </c>
-      <c r="I54" s="38" t="n">
+      <c r="I54" s="42" t="n">
         <v>231</v>
       </c>
-      <c r="J54" s="38" t="n">
+      <c r="J54" s="42" t="n">
         <v>235</v>
       </c>
-      <c r="K54" s="40">
+      <c r="K54" s="44">
         <f>J54*(J54/I54)</f>
         <v/>
       </c>
-      <c r="L54" s="41">
+      <c r="L54" s="45">
         <f>H54+K54</f>
         <v/>
       </c>
-      <c r="M54" s="38" t="n">
+      <c r="M54" s="42" t="n">
         <v>755</v>
       </c>
-      <c r="N54" s="38" t="n">
+      <c r="N54" s="42" t="n">
         <v>44</v>
       </c>
-      <c r="O54" s="42">
+      <c r="O54" s="46">
         <f>N54/M54</f>
         <v/>
       </c>
-      <c r="P54" s="41">
+      <c r="P54" s="45">
         <f>L54*O54</f>
         <v/>
       </c>
-      <c r="Q54" s="43" t="n">
+      <c r="Q54" s="47" t="n">
         <v>47</v>
       </c>
-      <c r="R54" s="44">
+      <c r="R54" s="48">
         <f>P54/Q54-1</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="45" t="inlineStr">
+      <c r="A55" s="49" t="inlineStr">
         <is>
           <t>GROUPE</t>
         </is>
       </c>
-      <c r="B55" s="30" t="n"/>
-      <c r="C55" s="30" t="n"/>
-      <c r="D55" s="30" t="n"/>
-      <c r="E55" s="30" t="n"/>
-      <c r="F55" s="30" t="n"/>
-      <c r="G55" s="30" t="n"/>
-      <c r="H55" s="30" t="n"/>
-      <c r="I55" s="30" t="n"/>
-      <c r="J55" s="30" t="n"/>
-      <c r="K55" s="30" t="n"/>
-      <c r="L55" s="46">
+      <c r="B55" s="50" t="n"/>
+      <c r="C55" s="50" t="n"/>
+      <c r="D55" s="50" t="n"/>
+      <c r="E55" s="50" t="n"/>
+      <c r="F55" s="50" t="n"/>
+      <c r="G55" s="50" t="n"/>
+      <c r="H55" s="50" t="n"/>
+      <c r="I55" s="50" t="n"/>
+      <c r="J55" s="50" t="n"/>
+      <c r="K55" s="50" t="n"/>
+      <c r="L55" s="51">
         <f>SUM(L41:L54)</f>
         <v/>
       </c>
-      <c r="M55" s="30" t="n"/>
-      <c r="N55" s="30" t="n"/>
-      <c r="O55" s="30" t="n"/>
-      <c r="P55" s="46">
+      <c r="M55" s="50" t="n"/>
+      <c r="N55" s="50" t="n"/>
+      <c r="O55" s="50" t="n"/>
+      <c r="P55" s="51">
         <f>SUM(P41:P54)</f>
         <v/>
       </c>
-      <c r="Q55" s="46">
+      <c r="Q55" s="51">
         <f>SUM(Q41:Q54)</f>
         <v/>
       </c>
-      <c r="R55" s="47">
+      <c r="R55" s="52">
         <f>P55/Q55-1</f>
         <v/>
       </c>
@@ -3173,481 +3319,481 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="48" t="inlineStr">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>Ipac Montpellier</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="25" t="n">
         <v>13581</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="25" t="n">
         <v>17870</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="25" t="n">
         <v>23514</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="22" t="n">
         <v>217</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="22" t="n">
         <v>237</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="22" t="n">
         <v>258</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="23">
         <f>SLOPE(LN(E8:G8),LN(B8:D8))</f>
         <v/>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="27">
         <f>G8*((1+$B$5)^H8-1)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>Ipac Nantes</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="25" t="n">
         <v>15937</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="25" t="n">
         <v>21082</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="25" t="n">
         <v>27889</v>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="22" t="n">
         <v>258</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="22" t="n">
         <v>281</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="22" t="n">
         <v>306</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="23">
         <f>SLOPE(LN(E9:G9),LN(B9:D9))</f>
         <v/>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="27">
         <f>G9*((1+$B$5)^H9-1)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="53" t="inlineStr">
         <is>
           <t>Ipac Rennes</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="25" t="n">
         <v>14022</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="25" t="n">
         <v>18403</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="25" t="n">
         <v>24152</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="22" t="n">
         <v>223</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="22" t="n">
         <v>243</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="22" t="n">
         <v>265</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="23">
         <f>SLOPE(LN(E10:G10),LN(B10:D10))</f>
         <v/>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="27">
         <f>G10*((1+$B$5)^H10-1)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+      <c r="A11" s="53" t="inlineStr">
         <is>
           <t>Iscom Lille</t>
         </is>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="25" t="n">
         <v>48495</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="25" t="n">
         <v>52768</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="25" t="n">
         <v>57418</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="22" t="n">
         <v>594</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="22" t="n">
         <v>612</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="22" t="n">
         <v>630</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="23">
         <f>SLOPE(LN(E11:G11),LN(B11:D11))</f>
         <v/>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="27">
         <f>G11*((1+$B$5)^H11-1)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="inlineStr">
+      <c r="A12" s="53" t="inlineStr">
         <is>
           <t>Iscom Paris</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="25" t="n">
         <v>52094</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="25" t="n">
         <v>57236</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="25" t="n">
         <v>62886</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="22" t="n">
         <v>650</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="22" t="n">
         <v>670</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="22" t="n">
         <v>690</v>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="23">
         <f>SLOPE(LN(E12:G12),LN(B12:D12))</f>
         <v/>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="27">
         <f>G12*((1+$B$5)^H12-1)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t>Iscom Toulouse</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="25" t="n">
         <v>46637</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="25" t="n">
         <v>50710</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="25" t="n">
         <v>55139</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="22" t="n">
         <v>570</v>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="22" t="n">
         <v>587</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="22" t="n">
         <v>605</v>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="23">
         <f>SLOPE(LN(E13:G13),LN(B13:D13))</f>
         <v/>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="27">
         <f>G13*((1+$B$5)^H13-1)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="48" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>MBway Bordeaux</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="25" t="n">
         <v>38877</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="25" t="n">
         <v>47246</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="25" t="n">
         <v>57418</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="22" t="n">
         <v>550</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="22" t="n">
         <v>589</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="22" t="n">
         <v>630</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="23">
         <f>SLOPE(LN(E14:G14),LN(B14:D14))</f>
         <v/>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="27">
         <f>G14*((1+$B$5)^H14-1)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="48" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>MBway Lyon</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="25" t="n">
         <v>43250</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="25" t="n">
         <v>53125</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="25" t="n">
         <v>65255</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="22" t="n">
         <v>626</v>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="22" t="n">
         <v>670</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="G15" s="22" t="n">
         <v>716</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="23">
         <f>SLOPE(LN(E15:G15),LN(B15:D15))</f>
         <v/>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="27">
         <f>G15*((1+$B$5)^H15-1)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="48" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>MBway Nantes</t>
         </is>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="25" t="n">
         <v>44771</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="25" t="n">
         <v>54502</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="25" t="n">
         <v>66349</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="22" t="n">
         <v>636</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="22" t="n">
         <v>680</v>
       </c>
-      <c r="G16" s="20" t="n">
+      <c r="G16" s="22" t="n">
         <v>728</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="23">
         <f>SLOPE(LN(E16:G16),LN(B16:D16))</f>
         <v/>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="27">
         <f>G16*((1+$B$5)^H16-1)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="48" t="inlineStr">
+      <c r="A17" s="53" t="inlineStr">
         <is>
           <t>MBway Paris</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="25" t="n">
         <v>41761</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="25" t="n">
         <v>52020</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="25" t="n">
         <v>64800</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="22" t="n">
         <v>621</v>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="22" t="n">
         <v>665</v>
       </c>
-      <c r="G17" s="20" t="n">
+      <c r="G17" s="22" t="n">
         <v>711</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="23">
         <f>SLOPE(LN(E17:G17),LN(B17:D17))</f>
         <v/>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="27">
         <f>G17*((1+$B$5)^H17-1)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="48" t="inlineStr">
+      <c r="A18" s="53" t="inlineStr">
         <is>
           <t>Pigier Bordeaux</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="25" t="n">
         <v>47760</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="25" t="n">
         <v>53273</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="25" t="n">
         <v>59423</v>
       </c>
-      <c r="E18" s="20" t="n">
+      <c r="E18" s="22" t="n">
         <v>603</v>
       </c>
-      <c r="F18" s="20" t="n">
+      <c r="F18" s="22" t="n">
         <v>627</v>
       </c>
-      <c r="G18" s="20" t="n">
+      <c r="G18" s="22" t="n">
         <v>652</v>
       </c>
-      <c r="H18" s="21">
+      <c r="H18" s="23">
         <f>SLOPE(LN(E18:G18),LN(B18:D18))</f>
         <v/>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="27">
         <f>G18*((1+$B$5)^H18-1)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="48" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>Pigier Lyon</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="25" t="n">
         <v>53439</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="25" t="n">
         <v>59953</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="25" t="n">
         <v>67261</v>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="22" t="n">
         <v>682</v>
       </c>
-      <c r="F19" s="20" t="n">
+      <c r="F19" s="22" t="n">
         <v>710</v>
       </c>
-      <c r="G19" s="20" t="n">
+      <c r="G19" s="22" t="n">
         <v>738</v>
       </c>
-      <c r="H19" s="21">
+      <c r="H19" s="23">
         <f>SLOPE(LN(E19:G19),LN(B19:D19))</f>
         <v/>
       </c>
-      <c r="I19" s="25">
+      <c r="I19" s="27">
         <f>G19*((1+$B$5)^H19-1)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="48" t="inlineStr">
+      <c r="A20" s="53" t="inlineStr">
         <is>
           <t>Tunon Lyon</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="25" t="n">
         <v>20221</v>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="25" t="n">
         <v>21550</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="25" t="n">
         <v>22967</v>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="22" t="n">
         <v>242</v>
       </c>
-      <c r="F20" s="20" t="n">
+      <c r="F20" s="22" t="n">
         <v>247</v>
       </c>
-      <c r="G20" s="20" t="n">
+      <c r="G20" s="22" t="n">
         <v>252</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="23">
         <f>SLOPE(LN(E20:G20),LN(B20:D20))</f>
         <v/>
       </c>
-      <c r="I20" s="25">
+      <c r="I20" s="27">
         <f>G20*((1+$B$5)^H20-1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="48" t="inlineStr">
+      <c r="A21" s="53" t="inlineStr">
         <is>
           <t>Tunon Paris</t>
         </is>
       </c>
-      <c r="B21" s="23" t="n">
+      <c r="B21" s="25" t="n">
         <v>19081</v>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="25" t="n">
         <v>20429</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="25" t="n">
         <v>21873</v>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="22" t="n">
         <v>231</v>
       </c>
-      <c r="F21" s="20" t="n">
+      <c r="F21" s="22" t="n">
         <v>235</v>
       </c>
-      <c r="G21" s="20" t="n">
+      <c r="G21" s="22" t="n">
         <v>240</v>
       </c>
-      <c r="H21" s="21">
+      <c r="H21" s="23">
         <f>SLOPE(LN(E21:G21),LN(B21:D21))</f>
         <v/>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="27">
         <f>G21*((1+$B$5)^H21-1)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="inlineStr">
+      <c r="A22" s="49" t="inlineStr">
         <is>
           <t>GROUPE</t>
         </is>
       </c>
-      <c r="B22" s="30" t="n"/>
-      <c r="C22" s="30" t="n"/>
-      <c r="D22" s="30" t="n"/>
-      <c r="E22" s="30" t="n"/>
-      <c r="F22" s="30" t="n"/>
-      <c r="G22" s="30" t="n"/>
-      <c r="H22" s="30" t="n"/>
-      <c r="I22" s="46">
+      <c r="B22" s="50" t="n"/>
+      <c r="C22" s="50" t="n"/>
+      <c r="D22" s="50" t="n"/>
+      <c r="E22" s="50" t="n"/>
+      <c r="F22" s="50" t="n"/>
+      <c r="G22" s="50" t="n"/>
+      <c r="H22" s="50" t="n"/>
+      <c r="I22" s="51">
         <f>SUM(I8:I21)</f>
         <v/>
       </c>
@@ -3660,7 +3806,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="36" t="inlineStr">
+      <c r="A26" s="40" t="inlineStr">
         <is>
           <t>Élasticité marque calculée sur 2024→2025 seulement, puis : organiques 2026 prédits = org.25 × (budget marque 26 ÷ budget marque 25) ^ élasticité(24→25).</t>
         </is>
@@ -3719,550 +3865,550 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="48" t="inlineStr">
+      <c r="A29" s="53" t="inlineStr">
         <is>
           <t>Ipac Montpellier</t>
         </is>
       </c>
-      <c r="B29" s="20" t="n">
+      <c r="B29" s="22" t="n">
         <v>217</v>
       </c>
-      <c r="C29" s="20" t="n">
+      <c r="C29" s="22" t="n">
         <v>237</v>
       </c>
-      <c r="D29" s="20" t="n">
+      <c r="D29" s="22" t="n">
         <v>13581</v>
       </c>
-      <c r="E29" s="20" t="n">
+      <c r="E29" s="22" t="n">
         <v>17870</v>
       </c>
-      <c r="F29" s="20" t="n">
+      <c r="F29" s="22" t="n">
         <v>23514</v>
       </c>
-      <c r="G29" s="49">
+      <c r="G29" s="54">
         <f>LN(C29/B29)/LN(E29/D29)</f>
         <v/>
       </c>
-      <c r="H29" s="50">
+      <c r="H29" s="55">
         <f>C29*(F29/E29)^G29</f>
         <v/>
       </c>
-      <c r="I29" s="25" t="n">
+      <c r="I29" s="27" t="n">
         <v>258</v>
       </c>
-      <c r="J29" s="51">
+      <c r="J29" s="56">
         <f>H29/I29-1</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="48" t="inlineStr">
+      <c r="A30" s="53" t="inlineStr">
         <is>
           <t>Ipac Nantes</t>
         </is>
       </c>
-      <c r="B30" s="20" t="n">
+      <c r="B30" s="22" t="n">
         <v>258</v>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="22" t="n">
         <v>281</v>
       </c>
-      <c r="D30" s="20" t="n">
+      <c r="D30" s="22" t="n">
         <v>15937</v>
       </c>
-      <c r="E30" s="20" t="n">
+      <c r="E30" s="22" t="n">
         <v>21082</v>
       </c>
-      <c r="F30" s="20" t="n">
+      <c r="F30" s="22" t="n">
         <v>27889</v>
       </c>
-      <c r="G30" s="49">
+      <c r="G30" s="54">
         <f>LN(C30/B30)/LN(E30/D30)</f>
         <v/>
       </c>
-      <c r="H30" s="50">
+      <c r="H30" s="55">
         <f>C30*(F30/E30)^G30</f>
         <v/>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="I30" s="27" t="n">
         <v>306</v>
       </c>
-      <c r="J30" s="51">
+      <c r="J30" s="56">
         <f>H30/I30-1</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="48" t="inlineStr">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>Ipac Rennes</t>
         </is>
       </c>
-      <c r="B31" s="20" t="n">
+      <c r="B31" s="22" t="n">
         <v>223</v>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="22" t="n">
         <v>243</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="22" t="n">
         <v>14022</v>
       </c>
-      <c r="E31" s="20" t="n">
+      <c r="E31" s="22" t="n">
         <v>18403</v>
       </c>
-      <c r="F31" s="20" t="n">
+      <c r="F31" s="22" t="n">
         <v>24152</v>
       </c>
-      <c r="G31" s="49">
+      <c r="G31" s="54">
         <f>LN(C31/B31)/LN(E31/D31)</f>
         <v/>
       </c>
-      <c r="H31" s="50">
+      <c r="H31" s="55">
         <f>C31*(F31/E31)^G31</f>
         <v/>
       </c>
-      <c r="I31" s="25" t="n">
+      <c r="I31" s="27" t="n">
         <v>265</v>
       </c>
-      <c r="J31" s="51">
+      <c r="J31" s="56">
         <f>H31/I31-1</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="48" t="inlineStr">
+      <c r="A32" s="53" t="inlineStr">
         <is>
           <t>Iscom Lille</t>
         </is>
       </c>
-      <c r="B32" s="20" t="n">
+      <c r="B32" s="22" t="n">
         <v>594</v>
       </c>
-      <c r="C32" s="20" t="n">
+      <c r="C32" s="22" t="n">
         <v>612</v>
       </c>
-      <c r="D32" s="20" t="n">
+      <c r="D32" s="22" t="n">
         <v>48495</v>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E32" s="22" t="n">
         <v>52768</v>
       </c>
-      <c r="F32" s="20" t="n">
+      <c r="F32" s="22" t="n">
         <v>57418</v>
       </c>
-      <c r="G32" s="49">
+      <c r="G32" s="54">
         <f>LN(C32/B32)/LN(E32/D32)</f>
         <v/>
       </c>
-      <c r="H32" s="50">
+      <c r="H32" s="55">
         <f>C32*(F32/E32)^G32</f>
         <v/>
       </c>
-      <c r="I32" s="25" t="n">
+      <c r="I32" s="27" t="n">
         <v>630</v>
       </c>
-      <c r="J32" s="51">
+      <c r="J32" s="56">
         <f>H32/I32-1</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="48" t="inlineStr">
+      <c r="A33" s="53" t="inlineStr">
         <is>
           <t>Iscom Paris</t>
         </is>
       </c>
-      <c r="B33" s="20" t="n">
+      <c r="B33" s="22" t="n">
         <v>650</v>
       </c>
-      <c r="C33" s="20" t="n">
+      <c r="C33" s="22" t="n">
         <v>670</v>
       </c>
-      <c r="D33" s="20" t="n">
+      <c r="D33" s="22" t="n">
         <v>52094</v>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E33" s="22" t="n">
         <v>57236</v>
       </c>
-      <c r="F33" s="20" t="n">
+      <c r="F33" s="22" t="n">
         <v>62886</v>
       </c>
-      <c r="G33" s="49">
+      <c r="G33" s="54">
         <f>LN(C33/B33)/LN(E33/D33)</f>
         <v/>
       </c>
-      <c r="H33" s="50">
+      <c r="H33" s="55">
         <f>C33*(F33/E33)^G33</f>
         <v/>
       </c>
-      <c r="I33" s="25" t="n">
+      <c r="I33" s="27" t="n">
         <v>690</v>
       </c>
-      <c r="J33" s="51">
+      <c r="J33" s="56">
         <f>H33/I33-1</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="48" t="inlineStr">
+      <c r="A34" s="53" t="inlineStr">
         <is>
           <t>Iscom Toulouse</t>
         </is>
       </c>
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="22" t="n">
         <v>570</v>
       </c>
-      <c r="C34" s="20" t="n">
+      <c r="C34" s="22" t="n">
         <v>587</v>
       </c>
-      <c r="D34" s="20" t="n">
+      <c r="D34" s="22" t="n">
         <v>46637</v>
       </c>
-      <c r="E34" s="20" t="n">
+      <c r="E34" s="22" t="n">
         <v>50710</v>
       </c>
-      <c r="F34" s="20" t="n">
+      <c r="F34" s="22" t="n">
         <v>55139</v>
       </c>
-      <c r="G34" s="49">
+      <c r="G34" s="54">
         <f>LN(C34/B34)/LN(E34/D34)</f>
         <v/>
       </c>
-      <c r="H34" s="50">
+      <c r="H34" s="55">
         <f>C34*(F34/E34)^G34</f>
         <v/>
       </c>
-      <c r="I34" s="25" t="n">
+      <c r="I34" s="27" t="n">
         <v>605</v>
       </c>
-      <c r="J34" s="51">
+      <c r="J34" s="56">
         <f>H34/I34-1</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="48" t="inlineStr">
+      <c r="A35" s="53" t="inlineStr">
         <is>
           <t>MBway Bordeaux</t>
         </is>
       </c>
-      <c r="B35" s="20" t="n">
+      <c r="B35" s="22" t="n">
         <v>550</v>
       </c>
-      <c r="C35" s="20" t="n">
+      <c r="C35" s="22" t="n">
         <v>589</v>
       </c>
-      <c r="D35" s="20" t="n">
+      <c r="D35" s="22" t="n">
         <v>38877</v>
       </c>
-      <c r="E35" s="20" t="n">
+      <c r="E35" s="22" t="n">
         <v>47246</v>
       </c>
-      <c r="F35" s="20" t="n">
+      <c r="F35" s="22" t="n">
         <v>57418</v>
       </c>
-      <c r="G35" s="49">
+      <c r="G35" s="54">
         <f>LN(C35/B35)/LN(E35/D35)</f>
         <v/>
       </c>
-      <c r="H35" s="50">
+      <c r="H35" s="55">
         <f>C35*(F35/E35)^G35</f>
         <v/>
       </c>
-      <c r="I35" s="25" t="n">
+      <c r="I35" s="27" t="n">
         <v>630</v>
       </c>
-      <c r="J35" s="51">
+      <c r="J35" s="56">
         <f>H35/I35-1</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="48" t="inlineStr">
+      <c r="A36" s="53" t="inlineStr">
         <is>
           <t>MBway Lyon</t>
         </is>
       </c>
-      <c r="B36" s="20" t="n">
+      <c r="B36" s="22" t="n">
         <v>626</v>
       </c>
-      <c r="C36" s="20" t="n">
+      <c r="C36" s="22" t="n">
         <v>670</v>
       </c>
-      <c r="D36" s="20" t="n">
+      <c r="D36" s="22" t="n">
         <v>43250</v>
       </c>
-      <c r="E36" s="20" t="n">
+      <c r="E36" s="22" t="n">
         <v>53125</v>
       </c>
-      <c r="F36" s="20" t="n">
+      <c r="F36" s="22" t="n">
         <v>65255</v>
       </c>
-      <c r="G36" s="49">
+      <c r="G36" s="54">
         <f>LN(C36/B36)/LN(E36/D36)</f>
         <v/>
       </c>
-      <c r="H36" s="50">
+      <c r="H36" s="55">
         <f>C36*(F36/E36)^G36</f>
         <v/>
       </c>
-      <c r="I36" s="25" t="n">
+      <c r="I36" s="27" t="n">
         <v>716</v>
       </c>
-      <c r="J36" s="51">
+      <c r="J36" s="56">
         <f>H36/I36-1</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="48" t="inlineStr">
+      <c r="A37" s="53" t="inlineStr">
         <is>
           <t>MBway Nantes</t>
         </is>
       </c>
-      <c r="B37" s="20" t="n">
+      <c r="B37" s="22" t="n">
         <v>636</v>
       </c>
-      <c r="C37" s="20" t="n">
+      <c r="C37" s="22" t="n">
         <v>680</v>
       </c>
-      <c r="D37" s="20" t="n">
+      <c r="D37" s="22" t="n">
         <v>44771</v>
       </c>
-      <c r="E37" s="20" t="n">
+      <c r="E37" s="22" t="n">
         <v>54502</v>
       </c>
-      <c r="F37" s="20" t="n">
+      <c r="F37" s="22" t="n">
         <v>66349</v>
       </c>
-      <c r="G37" s="49">
+      <c r="G37" s="54">
         <f>LN(C37/B37)/LN(E37/D37)</f>
         <v/>
       </c>
-      <c r="H37" s="50">
+      <c r="H37" s="55">
         <f>C37*(F37/E37)^G37</f>
         <v/>
       </c>
-      <c r="I37" s="25" t="n">
+      <c r="I37" s="27" t="n">
         <v>728</v>
       </c>
-      <c r="J37" s="51">
+      <c r="J37" s="56">
         <f>H37/I37-1</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="48" t="inlineStr">
+      <c r="A38" s="53" t="inlineStr">
         <is>
           <t>MBway Paris</t>
         </is>
       </c>
-      <c r="B38" s="20" t="n">
+      <c r="B38" s="22" t="n">
         <v>621</v>
       </c>
-      <c r="C38" s="20" t="n">
+      <c r="C38" s="22" t="n">
         <v>665</v>
       </c>
-      <c r="D38" s="20" t="n">
+      <c r="D38" s="22" t="n">
         <v>41761</v>
       </c>
-      <c r="E38" s="20" t="n">
+      <c r="E38" s="22" t="n">
         <v>52020</v>
       </c>
-      <c r="F38" s="20" t="n">
+      <c r="F38" s="22" t="n">
         <v>64800</v>
       </c>
-      <c r="G38" s="49">
+      <c r="G38" s="54">
         <f>LN(C38/B38)/LN(E38/D38)</f>
         <v/>
       </c>
-      <c r="H38" s="50">
+      <c r="H38" s="55">
         <f>C38*(F38/E38)^G38</f>
         <v/>
       </c>
-      <c r="I38" s="25" t="n">
+      <c r="I38" s="27" t="n">
         <v>711</v>
       </c>
-      <c r="J38" s="51">
+      <c r="J38" s="56">
         <f>H38/I38-1</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="48" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>Pigier Bordeaux</t>
         </is>
       </c>
-      <c r="B39" s="20" t="n">
+      <c r="B39" s="22" t="n">
         <v>603</v>
       </c>
-      <c r="C39" s="20" t="n">
+      <c r="C39" s="22" t="n">
         <v>627</v>
       </c>
-      <c r="D39" s="20" t="n">
+      <c r="D39" s="22" t="n">
         <v>47760</v>
       </c>
-      <c r="E39" s="20" t="n">
+      <c r="E39" s="22" t="n">
         <v>53273</v>
       </c>
-      <c r="F39" s="20" t="n">
+      <c r="F39" s="22" t="n">
         <v>59423</v>
       </c>
-      <c r="G39" s="49">
+      <c r="G39" s="54">
         <f>LN(C39/B39)/LN(E39/D39)</f>
         <v/>
       </c>
-      <c r="H39" s="50">
+      <c r="H39" s="55">
         <f>C39*(F39/E39)^G39</f>
         <v/>
       </c>
-      <c r="I39" s="25" t="n">
+      <c r="I39" s="27" t="n">
         <v>652</v>
       </c>
-      <c r="J39" s="51">
+      <c r="J39" s="56">
         <f>H39/I39-1</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="48" t="inlineStr">
+      <c r="A40" s="53" t="inlineStr">
         <is>
           <t>Pigier Lyon</t>
         </is>
       </c>
-      <c r="B40" s="20" t="n">
+      <c r="B40" s="22" t="n">
         <v>682</v>
       </c>
-      <c r="C40" s="20" t="n">
+      <c r="C40" s="22" t="n">
         <v>710</v>
       </c>
-      <c r="D40" s="20" t="n">
+      <c r="D40" s="22" t="n">
         <v>53439</v>
       </c>
-      <c r="E40" s="20" t="n">
+      <c r="E40" s="22" t="n">
         <v>59953</v>
       </c>
-      <c r="F40" s="20" t="n">
+      <c r="F40" s="22" t="n">
         <v>67261</v>
       </c>
-      <c r="G40" s="49">
+      <c r="G40" s="54">
         <f>LN(C40/B40)/LN(E40/D40)</f>
         <v/>
       </c>
-      <c r="H40" s="50">
+      <c r="H40" s="55">
         <f>C40*(F40/E40)^G40</f>
         <v/>
       </c>
-      <c r="I40" s="25" t="n">
+      <c r="I40" s="27" t="n">
         <v>738</v>
       </c>
-      <c r="J40" s="51">
+      <c r="J40" s="56">
         <f>H40/I40-1</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="48" t="inlineStr">
+      <c r="A41" s="53" t="inlineStr">
         <is>
           <t>Tunon Lyon</t>
         </is>
       </c>
-      <c r="B41" s="20" t="n">
+      <c r="B41" s="22" t="n">
         <v>242</v>
       </c>
-      <c r="C41" s="20" t="n">
+      <c r="C41" s="22" t="n">
         <v>247</v>
       </c>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="22" t="n">
         <v>20221</v>
       </c>
-      <c r="E41" s="20" t="n">
+      <c r="E41" s="22" t="n">
         <v>21550</v>
       </c>
-      <c r="F41" s="20" t="n">
+      <c r="F41" s="22" t="n">
         <v>22967</v>
       </c>
-      <c r="G41" s="49">
+      <c r="G41" s="54">
         <f>LN(C41/B41)/LN(E41/D41)</f>
         <v/>
       </c>
-      <c r="H41" s="50">
+      <c r="H41" s="55">
         <f>C41*(F41/E41)^G41</f>
         <v/>
       </c>
-      <c r="I41" s="25" t="n">
+      <c r="I41" s="27" t="n">
         <v>252</v>
       </c>
-      <c r="J41" s="51">
+      <c r="J41" s="56">
         <f>H41/I41-1</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="48" t="inlineStr">
+      <c r="A42" s="53" t="inlineStr">
         <is>
           <t>Tunon Paris</t>
         </is>
       </c>
-      <c r="B42" s="20" t="n">
+      <c r="B42" s="22" t="n">
         <v>231</v>
       </c>
-      <c r="C42" s="20" t="n">
+      <c r="C42" s="22" t="n">
         <v>235</v>
       </c>
-      <c r="D42" s="20" t="n">
+      <c r="D42" s="22" t="n">
         <v>19081</v>
       </c>
-      <c r="E42" s="20" t="n">
+      <c r="E42" s="22" t="n">
         <v>20429</v>
       </c>
-      <c r="F42" s="20" t="n">
+      <c r="F42" s="22" t="n">
         <v>21873</v>
       </c>
-      <c r="G42" s="49">
+      <c r="G42" s="54">
         <f>LN(C42/B42)/LN(E42/D42)</f>
         <v/>
       </c>
-      <c r="H42" s="50">
+      <c r="H42" s="55">
         <f>C42*(F42/E42)^G42</f>
         <v/>
       </c>
-      <c r="I42" s="25" t="n">
+      <c r="I42" s="27" t="n">
         <v>240</v>
       </c>
-      <c r="J42" s="51">
+      <c r="J42" s="56">
         <f>H42/I42-1</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="45" t="inlineStr">
+      <c r="A43" s="49" t="inlineStr">
         <is>
           <t>GROUPE</t>
         </is>
       </c>
-      <c r="B43" s="30" t="n"/>
-      <c r="C43" s="30" t="n"/>
-      <c r="D43" s="30" t="n"/>
-      <c r="E43" s="30" t="n"/>
-      <c r="F43" s="30" t="n"/>
-      <c r="G43" s="30" t="n"/>
-      <c r="H43" s="46">
+      <c r="B43" s="50" t="n"/>
+      <c r="C43" s="50" t="n"/>
+      <c r="D43" s="50" t="n"/>
+      <c r="E43" s="50" t="n"/>
+      <c r="F43" s="50" t="n"/>
+      <c r="G43" s="50" t="n"/>
+      <c r="H43" s="51">
         <f>SUM(H29:H42)</f>
         <v/>
       </c>
-      <c r="I43" s="46">
+      <c r="I43" s="51">
         <f>SUM(I29:I42)</f>
         <v/>
       </c>
-      <c r="J43" s="47">
+      <c r="J43" s="52">
         <f>H43/I43-1</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="52" t="inlineStr">
+      <c r="A45" s="57" t="inlineStr">
         <is>
           <t>Le moteur retrouve aussi les organiques 2026 sans les avoir vus. Les deux leviers (acquisition + marque) alimentent le MÊME funnel → inscrits → CA.</t>
         </is>

</xml_diff>